<commit_message>
Review 6 Problems 2/22/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C18A8B6-3CAC-422A-9D96-604ACC59EF11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CB13925-5363-4370-9ED4-8B511ACEE833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2359,32 +2359,6 @@
   </si>
   <si>
     <t>Infinite Sequences</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="14"/>
-        <color theme="1" tint="4.9989318521683403E-2"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Needs Review</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (76)</t>
-    </r>
   </si>
   <si>
     <t>Check your arguments</t>
@@ -2541,6 +2515,32 @@
   </si>
   <si>
     <t xml:space="preserve"> 1/2/2023</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="14"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Needs Review</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (77)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -4025,7 +4025,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>21</v>
@@ -4048,7 +4048,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>26</v>
@@ -7759,7 +7759,7 @@
       <c r="F163" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G163" s="50" t="s">
+      <c r="G163" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7782,7 +7782,7 @@
       <c r="F164" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G164" s="50" t="s">
+      <c r="G164" s="37" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7805,7 +7805,7 @@
       <c r="F165" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G165" s="50" t="s">
+      <c r="G165" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7828,7 +7828,7 @@
       <c r="F166" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G166" s="50" t="s">
+      <c r="G166" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       <c r="F167" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G167" s="50" t="s">
+      <c r="G167" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7862,7 +7862,7 @@
       <c r="B168" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C168" s="35" t="s">
+      <c r="C168" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D168" s="12" t="s">
@@ -7874,7 +7874,7 @@
       <c r="F168" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G168" s="50" t="s">
+      <c r="G168" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7885,7 +7885,7 @@
       <c r="B169" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C169" s="35" t="s">
+      <c r="C169" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D169" s="12" t="s">
@@ -7908,7 +7908,7 @@
       <c r="B170" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C170" s="35" t="s">
+      <c r="C170" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D170" s="12" t="s">
@@ -7931,7 +7931,7 @@
       <c r="B171" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C171" s="35" t="s">
+      <c r="C171" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D171" s="12" t="s">
@@ -7954,7 +7954,7 @@
       <c r="B172" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C172" s="35" t="s">
+      <c r="C172" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D172" s="12" t="s">
@@ -7977,7 +7977,7 @@
       <c r="B173" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C173" s="35" t="s">
+      <c r="C173" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D173" s="12" t="s">
@@ -8000,7 +8000,7 @@
       <c r="B174" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C174" s="35" t="s">
+      <c r="C174" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D174" s="12" t="s">
@@ -8023,7 +8023,7 @@
       <c r="B175" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C175" s="35" t="s">
+      <c r="C175" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D175" s="12" t="s">
@@ -8046,7 +8046,7 @@
       <c r="B176" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C176" s="35" t="s">
+      <c r="C176" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D176" s="12" t="s">
@@ -8092,7 +8092,7 @@
       <c r="B178" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C178" s="35" t="s">
+      <c r="C178" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D178" s="12" t="s">
@@ -8115,7 +8115,7 @@
       <c r="B179" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C179" s="35" t="s">
+      <c r="C179" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D179" s="12" t="s">
@@ -8138,7 +8138,7 @@
       <c r="B180" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C180" s="35" t="s">
+      <c r="C180" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D180" s="12" t="s">
@@ -8161,7 +8161,7 @@
       <c r="B181" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C181" s="35" t="s">
+      <c r="C181" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D181" s="12" t="s">
@@ -8184,7 +8184,7 @@
       <c r="B182" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C182" s="35" t="s">
+      <c r="C182" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D182" s="12" t="s">
@@ -8207,7 +8207,7 @@
       <c r="B183" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C183" s="35" t="s">
+      <c r="C183" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D183" s="12" t="s">
@@ -11174,7 +11174,7 @@
       <c r="B312" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C312" s="35" t="s">
+      <c r="C312" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D312" s="54">
@@ -11197,7 +11197,7 @@
       <c r="B313" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C313" s="35" t="s">
+      <c r="C313" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D313" s="54">
@@ -11266,7 +11266,7 @@
       <c r="B316" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C316" s="35" t="s">
+      <c r="C316" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D316" s="54">
@@ -13569,7 +13569,7 @@
       <c r="B416" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C416" s="35" t="s">
+      <c r="C416" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D416" s="54">
@@ -13592,7 +13592,7 @@
       <c r="B417" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C417" s="35" t="s">
+      <c r="C417" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D417" s="54">
@@ -13615,7 +13615,7 @@
       <c r="B418" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C418" s="35" t="s">
+      <c r="C418" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D418" s="54">
@@ -13638,7 +13638,7 @@
       <c r="B419" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C419" s="35" t="s">
+      <c r="C419" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D419" s="54">
@@ -13661,7 +13661,7 @@
       <c r="B420" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C420" s="35" t="s">
+      <c r="C420" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D420" s="54">
@@ -13684,7 +13684,7 @@
       <c r="B421" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C421" s="35" t="s">
+      <c r="C421" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D421" s="54">
@@ -13707,7 +13707,7 @@
       <c r="B422" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C422" s="35" t="s">
+      <c r="C422" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D422" s="54">
@@ -13730,7 +13730,7 @@
       <c r="B423" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C423" s="35" t="s">
+      <c r="C423" s="152" t="s">
         <v>13</v>
       </c>
       <c r="D423" s="54">
@@ -21205,7 +21205,7 @@
     </row>
     <row r="748" spans="1:7">
       <c r="A748" s="91" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B748" s="10" t="s">
         <v>22</v>
@@ -21228,7 +21228,7 @@
     </row>
     <row r="749" spans="1:7">
       <c r="A749" s="55" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="B749" s="10" t="s">
         <v>22</v>
@@ -21251,7 +21251,7 @@
     </row>
     <row r="750" spans="1:7">
       <c r="A750" s="73" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B750" s="10" t="s">
         <v>22</v>
@@ -21274,7 +21274,7 @@
     </row>
     <row r="751" spans="1:7">
       <c r="A751" s="82" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B751" s="10" t="s">
         <v>22</v>
@@ -21312,22 +21312,22 @@
     </row>
     <row r="757" spans="1:1" ht="18.5">
       <c r="A757" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="758" spans="1:1" ht="18.5">
       <c r="A758" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="759" spans="1:1" ht="18.5">
       <c r="A759" s="1" t="s">
-        <v>778</v>
+        <v>787</v>
       </c>
     </row>
     <row r="760" spans="1:1">
       <c r="A760" s="2" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="779" spans="1:6" ht="15.5">

</xml_diff>

<commit_message>
Review 10 Problems 2/25/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E343B889-0714-4081-A110-6462BC0A3A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4095C6A4-CA93-4B01-9C68-DA5DD2329F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8150,7 +8150,7 @@
       <c r="F180" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G180" s="50" t="s">
+      <c r="G180" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8173,7 +8173,7 @@
       <c r="F181" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G181" s="50" t="s">
+      <c r="G181" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8196,7 +8196,7 @@
       <c r="F182" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G182" s="50" t="s">
+      <c r="G182" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       <c r="F183" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G183" s="50" t="s">
+      <c r="G183" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8242,12 +8242,12 @@
       <c r="F184" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G184" s="50" t="s">
+      <c r="G184" s="11" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="185" spans="1:7">
-      <c r="A185" s="35" t="s">
+      <c r="A185" s="28" t="s">
         <v>154</v>
       </c>
       <c r="B185" s="7" t="s">
@@ -8265,7 +8265,7 @@
       <c r="F185" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G185" s="50" t="s">
+      <c r="G185" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8288,7 +8288,7 @@
       <c r="F186" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G186" s="50" t="s">
+      <c r="G186" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8311,7 +8311,7 @@
       <c r="F187" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G187" s="50" t="s">
+      <c r="G187" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8334,7 +8334,7 @@
       <c r="F188" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G188" s="50" t="s">
+      <c r="G188" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8357,7 +8357,7 @@
       <c r="F189" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G189" s="50" t="s">
+      <c r="G189" s="11" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 10 Problems 2/28/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4095C6A4-CA93-4B01-9C68-DA5DD2329F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB84ECF-D445-4664-B64B-6DC3A427119F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2539,7 +2539,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (78)</t>
+      <t xml:space="preserve"> (80)</t>
     </r>
   </si>
 </sst>
@@ -8380,7 +8380,7 @@
       <c r="F190" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G190" s="50" t="s">
+      <c r="G190" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8403,7 +8403,7 @@
       <c r="F191" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G191" s="50" t="s">
+      <c r="G191" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8426,7 +8426,7 @@
       <c r="F192" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G192" s="50" t="s">
+      <c r="G192" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8449,7 +8449,7 @@
       <c r="F193" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G193" s="50" t="s">
+      <c r="G193" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8472,7 +8472,7 @@
       <c r="F194" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G194" s="50" t="s">
+      <c r="G194" s="37" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8495,7 +8495,7 @@
       <c r="F195" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G195" s="50" t="s">
+      <c r="G195" s="37" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8518,7 +8518,7 @@
       <c r="F196" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G196" s="50" t="s">
+      <c r="G196" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8541,7 +8541,7 @@
       <c r="F197" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G197" s="50" t="s">
+      <c r="G197" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8564,7 +8564,7 @@
       <c r="F198" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G198" s="50" t="s">
+      <c r="G198" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8587,7 +8587,7 @@
       <c r="F199" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G199" s="50" t="s">
+      <c r="G199" s="11" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 5 Problems 3/1/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB84ECF-D445-4664-B64B-6DC3A427119F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D0B65A-AEDF-47AC-8926-7435C94D63D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8610,7 +8610,7 @@
       <c r="F200" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G200" s="50" t="s">
+      <c r="G200" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8633,7 +8633,7 @@
       <c r="F201" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G201" s="50" t="s">
+      <c r="G201" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8656,7 +8656,7 @@
       <c r="F202" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G202" s="50" t="s">
+      <c r="G202" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
       <c r="F203" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G203" s="50" t="s">
+      <c r="G203" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8702,7 +8702,7 @@
       <c r="F204" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G204" s="50" t="s">
+      <c r="G204" s="11" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 5 Problems 3/3/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D0B65A-AEDF-47AC-8926-7435C94D63D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45C6F9BE-BFD7-4538-A1CD-DD29286D5CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2539,7 +2539,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (80)</t>
+      <t xml:space="preserve"> (82)</t>
     </r>
   </si>
 </sst>
@@ -8725,7 +8725,7 @@
       <c r="F205" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G205" s="50" t="s">
+      <c r="G205" s="37" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8748,7 +8748,7 @@
       <c r="F206" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G206" s="50" t="s">
+      <c r="G206" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8771,7 +8771,7 @@
       <c r="F207" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G207" s="50" t="s">
+      <c r="G207" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8794,7 +8794,7 @@
       <c r="F208" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G208" s="50" t="s">
+      <c r="G208" s="11" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8817,7 +8817,7 @@
       <c r="F209" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="G209" s="50" t="s">
+      <c r="G209" s="37" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 4 Problems 4/15/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FFEC79-8B06-475E-A420-4685A40CDEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A978AB6-F0EF-41A6-A5B5-6DAD47154622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8946,7 +8946,7 @@
       <c r="F215" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G215" s="47" t="s">
+      <c r="G215" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8969,7 +8969,7 @@
       <c r="F216" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G216" s="47" t="s">
+      <c r="G216" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8992,7 +8992,7 @@
       <c r="F217" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G217" s="47" t="s">
+      <c r="G217" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       <c r="F218" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G218" s="47" t="s">
+      <c r="G218" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 5 Problems 4/21/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A978AB6-F0EF-41A6-A5B5-6DAD47154622}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADE3FAD-119A-4746-A012-0C8E18DCAADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9038,7 +9038,7 @@
       <c r="F219" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G219" s="47" t="s">
+      <c r="G219" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9061,7 +9061,7 @@
       <c r="F220" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G220" s="47" t="s">
+      <c r="G220" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9084,7 +9084,7 @@
       <c r="F221" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G221" s="47" t="s">
+      <c r="G221" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       <c r="F222" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G222" s="47" t="s">
+      <c r="G222" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9130,7 +9130,7 @@
       <c r="F223" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G223" s="47" t="s">
+      <c r="G223" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 6 Problems 4/22/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADE3FAD-119A-4746-A012-0C8E18DCAADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57382A24-AA65-46DB-B0B3-2C8D794C8AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3250,7 +3250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="151">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3441,9 +3441,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4489,7 +4486,7 @@
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="148" t="s">
+      <c r="A22" s="147" t="s">
         <v>14</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -5323,7 +5320,7 @@
       <c r="B58" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C58" s="149" t="s">
+      <c r="C58" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D58" s="10">
@@ -5346,7 +5343,7 @@
       <c r="B59" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C59" s="149" t="s">
+      <c r="C59" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D59" s="10">
@@ -5369,7 +5366,7 @@
       <c r="B60" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C60" s="149" t="s">
+      <c r="C60" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D60" s="10">
@@ -5392,7 +5389,7 @@
       <c r="B61" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C61" s="149" t="s">
+      <c r="C61" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D61" s="10">
@@ -5507,7 +5504,7 @@
       <c r="B66" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C66" s="149" t="s">
+      <c r="C66" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D66" s="10">
@@ -5530,7 +5527,7 @@
       <c r="B67" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C67" s="149" t="s">
+      <c r="C67" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D67" s="10">
@@ -7853,7 +7850,7 @@
       <c r="B168" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C168" s="149" t="s">
+      <c r="C168" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D168" s="10" t="s">
@@ -7876,7 +7873,7 @@
       <c r="B169" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C169" s="149" t="s">
+      <c r="C169" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D169" s="10" t="s">
@@ -7899,7 +7896,7 @@
       <c r="B170" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C170" s="149" t="s">
+      <c r="C170" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D170" s="10" t="s">
@@ -7922,7 +7919,7 @@
       <c r="B171" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C171" s="149" t="s">
+      <c r="C171" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D171" s="10" t="s">
@@ -7945,7 +7942,7 @@
       <c r="B172" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C172" s="149" t="s">
+      <c r="C172" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D172" s="10" t="s">
@@ -7968,7 +7965,7 @@
       <c r="B173" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C173" s="149" t="s">
+      <c r="C173" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D173" s="10" t="s">
@@ -7991,7 +7988,7 @@
       <c r="B174" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C174" s="149" t="s">
+      <c r="C174" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D174" s="10" t="s">
@@ -8014,7 +8011,7 @@
       <c r="B175" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C175" s="149" t="s">
+      <c r="C175" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D175" s="10" t="s">
@@ -8037,7 +8034,7 @@
       <c r="B176" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C176" s="149" t="s">
+      <c r="C176" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D176" s="10" t="s">
@@ -8083,7 +8080,7 @@
       <c r="B178" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C178" s="149" t="s">
+      <c r="C178" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D178" s="10" t="s">
@@ -8106,7 +8103,7 @@
       <c r="B179" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C179" s="149" t="s">
+      <c r="C179" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D179" s="10" t="s">
@@ -8129,7 +8126,7 @@
       <c r="B180" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C180" s="149" t="s">
+      <c r="C180" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D180" s="10" t="s">
@@ -8152,7 +8149,7 @@
       <c r="B181" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C181" s="149" t="s">
+      <c r="C181" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D181" s="10" t="s">
@@ -8175,7 +8172,7 @@
       <c r="B182" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C182" s="149" t="s">
+      <c r="C182" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D182" s="10" t="s">
@@ -8198,7 +8195,7 @@
       <c r="B183" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C183" s="149" t="s">
+      <c r="C183" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D183" s="10" t="s">
@@ -9153,7 +9150,7 @@
       <c r="F224" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G224" s="47" t="s">
+      <c r="G224" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9176,7 +9173,7 @@
       <c r="F225" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G225" s="47" t="s">
+      <c r="G225" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9199,7 +9196,7 @@
       <c r="F226" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G226" s="47" t="s">
+      <c r="G226" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9222,12 +9219,12 @@
       <c r="F227" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G227" s="47" t="s">
+      <c r="G227" s="9" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="228" spans="1:7">
-      <c r="A228" s="66" t="s">
+      <c r="A228" s="61" t="s">
         <v>195</v>
       </c>
       <c r="B228" s="8" t="s">
@@ -9245,12 +9242,12 @@
       <c r="F228" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G228" s="47" t="s">
+      <c r="G228" s="34" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="229" spans="1:7">
-      <c r="A229" s="67" t="s">
+      <c r="A229" s="66" t="s">
         <v>196</v>
       </c>
       <c r="B229" s="8" t="s">
@@ -9268,7 +9265,7 @@
       <c r="F229" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G229" s="47" t="s">
+      <c r="G229" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9365,7 +9362,7 @@
       </c>
     </row>
     <row r="234" spans="1:7">
-      <c r="A234" s="68" t="s">
+      <c r="A234" s="67" t="s">
         <v>199</v>
       </c>
       <c r="B234" s="8" t="s">
@@ -9457,7 +9454,7 @@
       </c>
     </row>
     <row r="238" spans="1:7">
-      <c r="A238" s="69" t="s">
+      <c r="A238" s="68" t="s">
         <v>203</v>
       </c>
       <c r="B238" s="8" t="s">
@@ -9480,7 +9477,7 @@
       </c>
     </row>
     <row r="239" spans="1:7">
-      <c r="A239" s="70" t="s">
+      <c r="A239" s="69" t="s">
         <v>204</v>
       </c>
       <c r="B239" s="8" t="s">
@@ -9664,7 +9661,7 @@
       </c>
     </row>
     <row r="247" spans="1:7">
-      <c r="A247" s="70" t="s">
+      <c r="A247" s="69" t="s">
         <v>730</v>
       </c>
       <c r="B247" s="8" t="s">
@@ -9733,7 +9730,7 @@
       </c>
     </row>
     <row r="250" spans="1:7">
-      <c r="A250" s="71" t="s">
+      <c r="A250" s="70" t="s">
         <v>215</v>
       </c>
       <c r="B250" s="8" t="s">
@@ -9756,7 +9753,7 @@
       </c>
     </row>
     <row r="251" spans="1:7">
-      <c r="A251" s="72" t="s">
+      <c r="A251" s="71" t="s">
         <v>216</v>
       </c>
       <c r="B251" s="8" t="s">
@@ -9779,7 +9776,7 @@
       </c>
     </row>
     <row r="252" spans="1:7">
-      <c r="A252" s="73" t="s">
+      <c r="A252" s="72" t="s">
         <v>217</v>
       </c>
       <c r="B252" s="8" t="s">
@@ -9802,7 +9799,7 @@
       </c>
     </row>
     <row r="253" spans="1:7">
-      <c r="A253" s="74" t="s">
+      <c r="A253" s="73" t="s">
         <v>218</v>
       </c>
       <c r="B253" s="8" t="s">
@@ -9825,7 +9822,7 @@
       </c>
     </row>
     <row r="254" spans="1:7">
-      <c r="A254" s="75" t="s">
+      <c r="A254" s="74" t="s">
         <v>219</v>
       </c>
       <c r="B254" s="8" t="s">
@@ -9848,7 +9845,7 @@
       </c>
     </row>
     <row r="255" spans="1:7">
-      <c r="A255" s="76" t="s">
+      <c r="A255" s="75" t="s">
         <v>220</v>
       </c>
       <c r="B255" s="8" t="s">
@@ -9871,7 +9868,7 @@
       </c>
     </row>
     <row r="256" spans="1:7">
-      <c r="A256" s="77" t="s">
+      <c r="A256" s="76" t="s">
         <v>221</v>
       </c>
       <c r="B256" s="8" t="s">
@@ -9894,7 +9891,7 @@
       </c>
     </row>
     <row r="257" spans="1:7">
-      <c r="A257" s="78" t="s">
+      <c r="A257" s="77" t="s">
         <v>222</v>
       </c>
       <c r="B257" s="8" t="s">
@@ -9917,7 +9914,7 @@
       </c>
     </row>
     <row r="258" spans="1:7">
-      <c r="A258" s="79" t="s">
+      <c r="A258" s="78" t="s">
         <v>223</v>
       </c>
       <c r="B258" s="8" t="s">
@@ -9940,7 +9937,7 @@
       </c>
     </row>
     <row r="259" spans="1:7">
-      <c r="A259" s="80" t="s">
+      <c r="A259" s="79" t="s">
         <v>224</v>
       </c>
       <c r="B259" s="8" t="s">
@@ -9963,7 +9960,7 @@
       </c>
     </row>
     <row r="260" spans="1:7">
-      <c r="A260" s="76" t="s">
+      <c r="A260" s="75" t="s">
         <v>225</v>
       </c>
       <c r="B260" s="8" t="s">
@@ -10032,7 +10029,7 @@
       </c>
     </row>
     <row r="263" spans="1:7">
-      <c r="A263" s="70" t="s">
+      <c r="A263" s="69" t="s">
         <v>228</v>
       </c>
       <c r="B263" s="8" t="s">
@@ -10193,7 +10190,7 @@
       </c>
     </row>
     <row r="270" spans="1:7">
-      <c r="A270" s="70" t="s">
+      <c r="A270" s="69" t="s">
         <v>235</v>
       </c>
       <c r="B270" s="8" t="s">
@@ -10239,7 +10236,7 @@
       </c>
     </row>
     <row r="272" spans="1:7">
-      <c r="A272" s="81" t="s">
+      <c r="A272" s="80" t="s">
         <v>743</v>
       </c>
       <c r="B272" s="8" t="s">
@@ -10262,7 +10259,7 @@
       </c>
     </row>
     <row r="273" spans="1:7">
-      <c r="A273" s="69" t="s">
+      <c r="A273" s="68" t="s">
         <v>237</v>
       </c>
       <c r="B273" s="8" t="s">
@@ -10308,7 +10305,7 @@
       </c>
     </row>
     <row r="275" spans="1:7">
-      <c r="A275" s="82" t="s">
+      <c r="A275" s="81" t="s">
         <v>239</v>
       </c>
       <c r="B275" s="8" t="s">
@@ -10446,7 +10443,7 @@
       </c>
     </row>
     <row r="281" spans="1:7">
-      <c r="A281" s="83" t="s">
+      <c r="A281" s="82" t="s">
         <v>247</v>
       </c>
       <c r="B281" s="22" t="s">
@@ -10768,7 +10765,7 @@
       </c>
     </row>
     <row r="295" spans="1:7">
-      <c r="A295" s="69" t="s">
+      <c r="A295" s="68" t="s">
         <v>260</v>
       </c>
       <c r="B295" s="8" t="s">
@@ -10814,7 +10811,7 @@
       </c>
     </row>
     <row r="297" spans="1:7">
-      <c r="A297" s="75" t="s">
+      <c r="A297" s="74" t="s">
         <v>266</v>
       </c>
       <c r="B297" s="8" t="s">
@@ -11165,7 +11162,7 @@
       <c r="B312" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C312" s="149" t="s">
+      <c r="C312" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D312" s="51">
@@ -11188,7 +11185,7 @@
       <c r="B313" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C313" s="149" t="s">
+      <c r="C313" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D313" s="51">
@@ -11257,7 +11254,7 @@
       <c r="B316" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C316" s="149" t="s">
+      <c r="C316" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D316" s="51">
@@ -11343,7 +11340,7 @@
       </c>
     </row>
     <row r="320" spans="1:7">
-      <c r="A320" s="73" t="s">
+      <c r="A320" s="72" t="s">
         <v>342</v>
       </c>
       <c r="B320" s="8" t="s">
@@ -11458,7 +11455,7 @@
       </c>
     </row>
     <row r="325" spans="1:7">
-      <c r="A325" s="75" t="s">
+      <c r="A325" s="74" t="s">
         <v>348</v>
       </c>
       <c r="B325" s="8" t="s">
@@ -12056,7 +12053,7 @@
       </c>
     </row>
     <row r="351" spans="1:7">
-      <c r="A351" s="73" t="s">
+      <c r="A351" s="72" t="s">
         <v>371</v>
       </c>
       <c r="B351" s="8" t="s">
@@ -12148,7 +12145,7 @@
       </c>
     </row>
     <row r="355" spans="1:7">
-      <c r="A355" s="79" t="s">
+      <c r="A355" s="78" t="s">
         <v>375</v>
       </c>
       <c r="B355" s="8" t="s">
@@ -12332,7 +12329,7 @@
       </c>
     </row>
     <row r="363" spans="1:7">
-      <c r="A363" s="84" t="s">
+      <c r="A363" s="83" t="s">
         <v>383</v>
       </c>
       <c r="B363" s="22" t="s">
@@ -12424,7 +12421,7 @@
       </c>
     </row>
     <row r="367" spans="1:7">
-      <c r="A367" s="85" t="s">
+      <c r="A367" s="84" t="s">
         <v>387</v>
       </c>
       <c r="B367" s="8" t="s">
@@ -12470,7 +12467,7 @@
       </c>
     </row>
     <row r="369" spans="1:7">
-      <c r="A369" s="85" t="s">
+      <c r="A369" s="84" t="s">
         <v>389</v>
       </c>
       <c r="B369" s="8" t="s">
@@ -12516,7 +12513,7 @@
       </c>
     </row>
     <row r="371" spans="1:7">
-      <c r="A371" s="69" t="s">
+      <c r="A371" s="68" t="s">
         <v>391</v>
       </c>
       <c r="B371" s="8" t="s">
@@ -12585,7 +12582,7 @@
       </c>
     </row>
     <row r="374" spans="1:7">
-      <c r="A374" s="86" t="s">
+      <c r="A374" s="85" t="s">
         <v>394</v>
       </c>
       <c r="B374" s="22" t="s">
@@ -12631,7 +12628,7 @@
       </c>
     </row>
     <row r="376" spans="1:7">
-      <c r="A376" s="87" t="s">
+      <c r="A376" s="86" t="s">
         <v>395</v>
       </c>
       <c r="B376" s="8" t="s">
@@ -12815,7 +12812,7 @@
       </c>
     </row>
     <row r="384" spans="1:7">
-      <c r="A384" s="88" t="s">
+      <c r="A384" s="87" t="s">
         <v>403</v>
       </c>
       <c r="B384" s="8" t="s">
@@ -12838,7 +12835,7 @@
       </c>
     </row>
     <row r="385" spans="1:8">
-      <c r="A385" s="89" t="s">
+      <c r="A385" s="88" t="s">
         <v>404</v>
       </c>
       <c r="B385" s="8" t="s">
@@ -12930,7 +12927,7 @@
       </c>
     </row>
     <row r="389" spans="1:8">
-      <c r="A389" s="70" t="s">
+      <c r="A389" s="69" t="s">
         <v>408</v>
       </c>
       <c r="B389" s="8" t="s">
@@ -12976,7 +12973,7 @@
       </c>
     </row>
     <row r="391" spans="1:8">
-      <c r="A391" s="90" t="s">
+      <c r="A391" s="89" t="s">
         <v>410</v>
       </c>
       <c r="B391" s="8" t="s">
@@ -13046,7 +13043,7 @@
       </c>
     </row>
     <row r="394" spans="1:8">
-      <c r="A394" s="91" t="s">
+      <c r="A394" s="90" t="s">
         <v>413</v>
       </c>
       <c r="B394" s="22" t="s">
@@ -13069,7 +13066,7 @@
       </c>
     </row>
     <row r="395" spans="1:8">
-      <c r="A395" s="92" t="s">
+      <c r="A395" s="91" t="s">
         <v>414</v>
       </c>
       <c r="B395" s="8" t="s">
@@ -13162,7 +13159,7 @@
       </c>
     </row>
     <row r="399" spans="1:8">
-      <c r="A399" s="93" t="s">
+      <c r="A399" s="92" t="s">
         <v>418</v>
       </c>
       <c r="B399" s="8" t="s">
@@ -13231,7 +13228,7 @@
       </c>
     </row>
     <row r="402" spans="1:8">
-      <c r="A402" s="94" t="s">
+      <c r="A402" s="93" t="s">
         <v>421</v>
       </c>
       <c r="B402" s="8" t="s">
@@ -13300,7 +13297,7 @@
       </c>
     </row>
     <row r="405" spans="1:8">
-      <c r="A405" s="95" t="s">
+      <c r="A405" s="94" t="s">
         <v>424</v>
       </c>
       <c r="B405" s="8" t="s">
@@ -13439,7 +13436,7 @@
       </c>
     </row>
     <row r="411" spans="1:8">
-      <c r="A411" s="75" t="s">
+      <c r="A411" s="74" t="s">
         <v>430</v>
       </c>
       <c r="B411" s="8" t="s">
@@ -13508,7 +13505,7 @@
       </c>
     </row>
     <row r="414" spans="1:8">
-      <c r="A414" s="75" t="s">
+      <c r="A414" s="74" t="s">
         <v>657</v>
       </c>
       <c r="B414" s="8" t="s">
@@ -13554,13 +13551,13 @@
       </c>
     </row>
     <row r="416" spans="1:8">
-      <c r="A416" s="96" t="s">
+      <c r="A416" s="95" t="s">
         <v>434</v>
       </c>
       <c r="B416" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C416" s="149" t="s">
+      <c r="C416" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D416" s="51">
@@ -13577,13 +13574,13 @@
       </c>
     </row>
     <row r="417" spans="1:7">
-      <c r="A417" s="97" t="s">
+      <c r="A417" s="96" t="s">
         <v>435</v>
       </c>
       <c r="B417" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C417" s="149" t="s">
+      <c r="C417" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D417" s="51">
@@ -13600,13 +13597,13 @@
       </c>
     </row>
     <row r="418" spans="1:7">
-      <c r="A418" s="86" t="s">
+      <c r="A418" s="85" t="s">
         <v>436</v>
       </c>
       <c r="B418" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C418" s="149" t="s">
+      <c r="C418" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D418" s="51">
@@ -13623,13 +13620,13 @@
       </c>
     </row>
     <row r="419" spans="1:7">
-      <c r="A419" s="91" t="s">
+      <c r="A419" s="90" t="s">
         <v>437</v>
       </c>
       <c r="B419" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C419" s="149" t="s">
+      <c r="C419" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D419" s="51">
@@ -13646,13 +13643,13 @@
       </c>
     </row>
     <row r="420" spans="1:7">
-      <c r="A420" s="98" t="s">
+      <c r="A420" s="97" t="s">
         <v>438</v>
       </c>
       <c r="B420" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C420" s="149" t="s">
+      <c r="C420" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D420" s="51">
@@ -13669,13 +13666,13 @@
       </c>
     </row>
     <row r="421" spans="1:7">
-      <c r="A421" s="99" t="s">
+      <c r="A421" s="98" t="s">
         <v>727</v>
       </c>
       <c r="B421" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C421" s="149" t="s">
+      <c r="C421" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D421" s="51">
@@ -13692,13 +13689,13 @@
       </c>
     </row>
     <row r="422" spans="1:7">
-      <c r="A422" s="96" t="s">
+      <c r="A422" s="95" t="s">
         <v>728</v>
       </c>
       <c r="B422" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C422" s="149" t="s">
+      <c r="C422" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D422" s="51">
@@ -13715,13 +13712,13 @@
       </c>
     </row>
     <row r="423" spans="1:7">
-      <c r="A423" s="100" t="s">
+      <c r="A423" s="99" t="s">
         <v>729</v>
       </c>
       <c r="B423" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C423" s="149" t="s">
+      <c r="C423" s="148" t="s">
         <v>13</v>
       </c>
       <c r="D423" s="51">
@@ -13738,7 +13735,7 @@
       </c>
     </row>
     <row r="424" spans="1:7">
-      <c r="A424" s="85" t="s">
+      <c r="A424" s="84" t="s">
         <v>439</v>
       </c>
       <c r="B424" s="8" t="s">
@@ -13761,7 +13758,7 @@
       </c>
     </row>
     <row r="425" spans="1:7">
-      <c r="A425" s="87" t="s">
+      <c r="A425" s="86" t="s">
         <v>440</v>
       </c>
       <c r="B425" s="8" t="s">
@@ -13830,7 +13827,7 @@
       </c>
     </row>
     <row r="428" spans="1:7">
-      <c r="A428" s="101" t="s">
+      <c r="A428" s="100" t="s">
         <v>443</v>
       </c>
       <c r="B428" s="4" t="s">
@@ -13853,7 +13850,7 @@
       </c>
     </row>
     <row r="429" spans="1:7">
-      <c r="A429" s="98" t="s">
+      <c r="A429" s="97" t="s">
         <v>444</v>
       </c>
       <c r="B429" s="8" t="s">
@@ -13922,7 +13919,7 @@
       </c>
     </row>
     <row r="432" spans="1:7">
-      <c r="A432" s="70" t="s">
+      <c r="A432" s="69" t="s">
         <v>447</v>
       </c>
       <c r="B432" s="8" t="s">
@@ -13968,7 +13965,7 @@
       </c>
     </row>
     <row r="434" spans="1:7">
-      <c r="A434" s="102" t="s">
+      <c r="A434" s="101" t="s">
         <v>449</v>
       </c>
       <c r="B434" s="4" t="s">
@@ -14037,7 +14034,7 @@
       </c>
     </row>
     <row r="437" spans="1:7">
-      <c r="A437" s="103" t="s">
+      <c r="A437" s="102" t="s">
         <v>453</v>
       </c>
       <c r="B437" s="4" t="s">
@@ -14083,7 +14080,7 @@
       </c>
     </row>
     <row r="439" spans="1:7">
-      <c r="A439" s="104" t="s">
+      <c r="A439" s="103" t="s">
         <v>455</v>
       </c>
       <c r="B439" s="8" t="s">
@@ -14106,7 +14103,7 @@
       </c>
     </row>
     <row r="440" spans="1:7">
-      <c r="A440" s="99" t="s">
+      <c r="A440" s="98" t="s">
         <v>456</v>
       </c>
       <c r="B440" s="8" t="s">
@@ -14152,7 +14149,7 @@
       </c>
     </row>
     <row r="442" spans="1:7">
-      <c r="A442" s="105" t="s">
+      <c r="A442" s="104" t="s">
         <v>458</v>
       </c>
       <c r="B442" s="8" t="s">
@@ -14198,7 +14195,7 @@
       </c>
     </row>
     <row r="444" spans="1:7">
-      <c r="A444" s="91" t="s">
+      <c r="A444" s="90" t="s">
         <v>460</v>
       </c>
       <c r="B444" s="8" t="s">
@@ -14221,7 +14218,7 @@
       </c>
     </row>
     <row r="445" spans="1:7">
-      <c r="A445" s="106" t="s">
+      <c r="A445" s="105" t="s">
         <v>461</v>
       </c>
       <c r="B445" s="8" t="s">
@@ -14290,7 +14287,7 @@
       </c>
     </row>
     <row r="448" spans="1:7">
-      <c r="A448" s="87" t="s">
+      <c r="A448" s="86" t="s">
         <v>464</v>
       </c>
       <c r="B448" s="8" t="s">
@@ -14313,7 +14310,7 @@
       </c>
     </row>
     <row r="449" spans="1:7">
-      <c r="A449" s="100" t="s">
+      <c r="A449" s="99" t="s">
         <v>465</v>
       </c>
       <c r="B449" s="8" t="s">
@@ -14336,7 +14333,7 @@
       </c>
     </row>
     <row r="450" spans="1:7">
-      <c r="A450" s="107" t="s">
+      <c r="A450" s="106" t="s">
         <v>466</v>
       </c>
       <c r="B450" s="8" t="s">
@@ -14382,7 +14379,7 @@
       </c>
     </row>
     <row r="452" spans="1:7">
-      <c r="A452" s="96" t="s">
+      <c r="A452" s="95" t="s">
         <v>468</v>
       </c>
       <c r="B452" s="8" t="s">
@@ -14405,7 +14402,7 @@
       </c>
     </row>
     <row r="453" spans="1:7">
-      <c r="A453" s="84" t="s">
+      <c r="A453" s="83" t="s">
         <v>469</v>
       </c>
       <c r="B453" s="8" t="s">
@@ -14428,7 +14425,7 @@
       </c>
     </row>
     <row r="454" spans="1:7">
-      <c r="A454" s="79" t="s">
+      <c r="A454" s="78" t="s">
         <v>470</v>
       </c>
       <c r="B454" s="8" t="s">
@@ -14474,7 +14471,7 @@
       </c>
     </row>
     <row r="456" spans="1:7">
-      <c r="A456" s="103" t="s">
+      <c r="A456" s="102" t="s">
         <v>472</v>
       </c>
       <c r="B456" s="8" t="s">
@@ -14497,7 +14494,7 @@
       </c>
     </row>
     <row r="457" spans="1:7">
-      <c r="A457" s="87" t="s">
+      <c r="A457" s="86" t="s">
         <v>473</v>
       </c>
       <c r="B457" s="8" t="s">
@@ -14520,7 +14517,7 @@
       </c>
     </row>
     <row r="458" spans="1:7">
-      <c r="A458" s="98" t="s">
+      <c r="A458" s="97" t="s">
         <v>474</v>
       </c>
       <c r="B458" s="8" t="s">
@@ -14543,7 +14540,7 @@
       </c>
     </row>
     <row r="459" spans="1:7">
-      <c r="A459" s="103" t="s">
+      <c r="A459" s="102" t="s">
         <v>475</v>
       </c>
       <c r="B459" s="8" t="s">
@@ -14589,7 +14586,7 @@
       </c>
     </row>
     <row r="461" spans="1:7">
-      <c r="A461" s="86" t="s">
+      <c r="A461" s="85" t="s">
         <v>477</v>
       </c>
       <c r="B461" s="8" t="s">
@@ -14612,7 +14609,7 @@
       </c>
     </row>
     <row r="462" spans="1:7">
-      <c r="A462" s="108" t="s">
+      <c r="A462" s="107" t="s">
         <v>478</v>
       </c>
       <c r="B462" s="8" t="s">
@@ -14658,7 +14655,7 @@
       </c>
     </row>
     <row r="464" spans="1:7">
-      <c r="A464" s="109" t="s">
+      <c r="A464" s="108" t="s">
         <v>480</v>
       </c>
       <c r="B464" s="8" t="s">
@@ -14704,7 +14701,7 @@
       </c>
     </row>
     <row r="466" spans="1:7">
-      <c r="A466" s="110" t="s">
+      <c r="A466" s="109" t="s">
         <v>482</v>
       </c>
       <c r="B466" s="8" t="s">
@@ -14727,7 +14724,7 @@
       </c>
     </row>
     <row r="467" spans="1:7">
-      <c r="A467" s="97" t="s">
+      <c r="A467" s="96" t="s">
         <v>483</v>
       </c>
       <c r="B467" s="8" t="s">
@@ -14750,7 +14747,7 @@
       </c>
     </row>
     <row r="468" spans="1:7">
-      <c r="A468" s="98" t="s">
+      <c r="A468" s="97" t="s">
         <v>484</v>
       </c>
       <c r="B468" s="8" t="s">
@@ -14773,7 +14770,7 @@
       </c>
     </row>
     <row r="469" spans="1:7">
-      <c r="A469" s="108" t="s">
+      <c r="A469" s="107" t="s">
         <v>485</v>
       </c>
       <c r="B469" s="8" t="s">
@@ -14819,7 +14816,7 @@
       </c>
     </row>
     <row r="471" spans="1:7">
-      <c r="A471" s="111" t="s">
+      <c r="A471" s="110" t="s">
         <v>487</v>
       </c>
       <c r="B471" s="8" t="s">
@@ -14911,7 +14908,7 @@
       </c>
     </row>
     <row r="475" spans="1:7">
-      <c r="A475" s="77" t="s">
+      <c r="A475" s="76" t="s">
         <v>491</v>
       </c>
       <c r="B475" s="8" t="s">
@@ -14934,7 +14931,7 @@
       </c>
     </row>
     <row r="476" spans="1:7">
-      <c r="A476" s="82" t="s">
+      <c r="A476" s="81" t="s">
         <v>492</v>
       </c>
       <c r="B476" s="8" t="s">
@@ -14980,7 +14977,7 @@
       </c>
     </row>
     <row r="478" spans="1:7">
-      <c r="A478" s="98" t="s">
+      <c r="A478" s="97" t="s">
         <v>494</v>
       </c>
       <c r="B478" s="8" t="s">
@@ -15003,7 +15000,7 @@
       </c>
     </row>
     <row r="479" spans="1:7">
-      <c r="A479" s="75" t="s">
+      <c r="A479" s="74" t="s">
         <v>495</v>
       </c>
       <c r="B479" s="8" t="s">
@@ -15026,7 +15023,7 @@
       </c>
     </row>
     <row r="480" spans="1:7">
-      <c r="A480" s="109" t="s">
+      <c r="A480" s="108" t="s">
         <v>496</v>
       </c>
       <c r="B480" s="8" t="s">
@@ -15095,7 +15092,7 @@
       </c>
     </row>
     <row r="483" spans="1:7">
-      <c r="A483" s="86" t="s">
+      <c r="A483" s="85" t="s">
         <v>499</v>
       </c>
       <c r="B483" s="8" t="s">
@@ -15118,7 +15115,7 @@
       </c>
     </row>
     <row r="484" spans="1:7">
-      <c r="A484" s="112" t="s">
+      <c r="A484" s="111" t="s">
         <v>500</v>
       </c>
       <c r="B484" s="8" t="s">
@@ -15141,7 +15138,7 @@
       </c>
     </row>
     <row r="485" spans="1:7">
-      <c r="A485" s="113" t="s">
+      <c r="A485" s="112" t="s">
         <v>501</v>
       </c>
       <c r="B485" s="8" t="s">
@@ -15164,7 +15161,7 @@
       </c>
     </row>
     <row r="486" spans="1:7">
-      <c r="A486" s="108" t="s">
+      <c r="A486" s="107" t="s">
         <v>502</v>
       </c>
       <c r="B486" s="8" t="s">
@@ -15210,7 +15207,7 @@
       </c>
     </row>
     <row r="488" spans="1:7">
-      <c r="A488" s="114" t="s">
+      <c r="A488" s="113" t="s">
         <v>504</v>
       </c>
       <c r="B488" s="8" t="s">
@@ -15233,7 +15230,7 @@
       </c>
     </row>
     <row r="489" spans="1:7">
-      <c r="A489" s="75" t="s">
+      <c r="A489" s="74" t="s">
         <v>505</v>
       </c>
       <c r="B489" s="8" t="s">
@@ -15256,7 +15253,7 @@
       </c>
     </row>
     <row r="490" spans="1:7">
-      <c r="A490" s="88" t="s">
+      <c r="A490" s="87" t="s">
         <v>506</v>
       </c>
       <c r="B490" s="8" t="s">
@@ -15279,7 +15276,7 @@
       </c>
     </row>
     <row r="491" spans="1:7">
-      <c r="A491" s="108" t="s">
+      <c r="A491" s="107" t="s">
         <v>507</v>
       </c>
       <c r="B491" s="8" t="s">
@@ -15302,7 +15299,7 @@
       </c>
     </row>
     <row r="492" spans="1:7">
-      <c r="A492" s="97" t="s">
+      <c r="A492" s="96" t="s">
         <v>508</v>
       </c>
       <c r="B492" s="8" t="s">
@@ -15348,7 +15345,7 @@
       </c>
     </row>
     <row r="494" spans="1:7">
-      <c r="A494" s="92" t="s">
+      <c r="A494" s="91" t="s">
         <v>510</v>
       </c>
       <c r="B494" s="8" t="s">
@@ -15371,7 +15368,7 @@
       </c>
     </row>
     <row r="495" spans="1:7">
-      <c r="A495" s="91" t="s">
+      <c r="A495" s="90" t="s">
         <v>511</v>
       </c>
       <c r="B495" s="8" t="s">
@@ -15440,7 +15437,7 @@
       </c>
     </row>
     <row r="498" spans="1:8">
-      <c r="A498" s="98" t="s">
+      <c r="A498" s="97" t="s">
         <v>514</v>
       </c>
       <c r="B498" s="8" t="s">
@@ -15463,7 +15460,7 @@
       </c>
     </row>
     <row r="499" spans="1:8">
-      <c r="A499" s="86" t="s">
+      <c r="A499" s="85" t="s">
         <v>515</v>
       </c>
       <c r="B499" s="8" t="s">
@@ -15486,7 +15483,7 @@
       </c>
     </row>
     <row r="500" spans="1:8">
-      <c r="A500" s="103" t="s">
+      <c r="A500" s="102" t="s">
         <v>516</v>
       </c>
       <c r="B500" s="8" t="s">
@@ -15509,7 +15506,7 @@
       </c>
     </row>
     <row r="501" spans="1:8">
-      <c r="A501" s="99" t="s">
+      <c r="A501" s="98" t="s">
         <v>517</v>
       </c>
       <c r="B501" s="8" t="s">
@@ -15532,7 +15529,7 @@
       </c>
     </row>
     <row r="502" spans="1:8">
-      <c r="A502" s="115" t="s">
+      <c r="A502" s="114" t="s">
         <v>518</v>
       </c>
       <c r="B502" s="8" t="s">
@@ -15555,7 +15552,7 @@
       </c>
     </row>
     <row r="503" spans="1:8">
-      <c r="A503" s="108" t="s">
+      <c r="A503" s="107" t="s">
         <v>520</v>
       </c>
       <c r="B503" s="8" t="s">
@@ -15578,7 +15575,7 @@
       </c>
     </row>
     <row r="504" spans="1:8">
-      <c r="A504" s="93" t="s">
+      <c r="A504" s="92" t="s">
         <v>519</v>
       </c>
       <c r="B504" s="8" t="s">
@@ -15601,7 +15598,7 @@
       </c>
     </row>
     <row r="505" spans="1:8">
-      <c r="A505" s="109" t="s">
+      <c r="A505" s="108" t="s">
         <v>521</v>
       </c>
       <c r="B505" s="8" t="s">
@@ -15625,7 +15622,7 @@
       <c r="H505" s="15"/>
     </row>
     <row r="506" spans="1:8">
-      <c r="A506" s="111" t="s">
+      <c r="A506" s="110" t="s">
         <v>522</v>
       </c>
       <c r="B506" s="8" t="s">
@@ -15648,7 +15645,7 @@
       </c>
     </row>
     <row r="507" spans="1:8">
-      <c r="A507" s="92" t="s">
+      <c r="A507" s="91" t="s">
         <v>523</v>
       </c>
       <c r="B507" s="8" t="s">
@@ -15671,7 +15668,7 @@
       </c>
     </row>
     <row r="508" spans="1:8">
-      <c r="A508" s="75" t="s">
+      <c r="A508" s="74" t="s">
         <v>524</v>
       </c>
       <c r="B508" s="8" t="s">
@@ -15694,7 +15691,7 @@
       </c>
     </row>
     <row r="509" spans="1:8">
-      <c r="A509" s="99" t="s">
+      <c r="A509" s="98" t="s">
         <v>524</v>
       </c>
       <c r="B509" s="8" t="s">
@@ -15809,7 +15806,7 @@
       </c>
     </row>
     <row r="514" spans="1:7">
-      <c r="A514" s="103" t="s">
+      <c r="A514" s="102" t="s">
         <v>529</v>
       </c>
       <c r="B514" s="8" t="s">
@@ -15832,7 +15829,7 @@
       </c>
     </row>
     <row r="515" spans="1:7">
-      <c r="A515" s="107" t="s">
+      <c r="A515" s="106" t="s">
         <v>530</v>
       </c>
       <c r="B515" s="8" t="s">
@@ -15855,7 +15852,7 @@
       </c>
     </row>
     <row r="516" spans="1:7">
-      <c r="A516" s="108" t="s">
+      <c r="A516" s="107" t="s">
         <v>531</v>
       </c>
       <c r="B516" s="8" t="s">
@@ -15878,7 +15875,7 @@
       </c>
     </row>
     <row r="517" spans="1:7">
-      <c r="A517" s="101" t="s">
+      <c r="A517" s="100" t="s">
         <v>532</v>
       </c>
       <c r="B517" s="8" t="s">
@@ -15901,7 +15898,7 @@
       </c>
     </row>
     <row r="518" spans="1:7">
-      <c r="A518" s="74" t="s">
+      <c r="A518" s="73" t="s">
         <v>533</v>
       </c>
       <c r="B518" s="8" t="s">
@@ -15924,7 +15921,7 @@
       </c>
     </row>
     <row r="519" spans="1:7">
-      <c r="A519" s="103" t="s">
+      <c r="A519" s="102" t="s">
         <v>534</v>
       </c>
       <c r="B519" s="8" t="s">
@@ -16039,7 +16036,7 @@
       </c>
     </row>
     <row r="524" spans="1:7">
-      <c r="A524" s="85" t="s">
+      <c r="A524" s="84" t="s">
         <v>539</v>
       </c>
       <c r="B524" s="8" t="s">
@@ -16154,7 +16151,7 @@
       </c>
     </row>
     <row r="529" spans="1:8">
-      <c r="A529" s="116" t="s">
+      <c r="A529" s="115" t="s">
         <v>544</v>
       </c>
       <c r="B529" s="8" t="s">
@@ -16200,7 +16197,7 @@
       </c>
     </row>
     <row r="531" spans="1:8">
-      <c r="A531" s="97" t="s">
+      <c r="A531" s="96" t="s">
         <v>546</v>
       </c>
       <c r="B531" s="8" t="s">
@@ -16221,10 +16218,10 @@
       <c r="G531" s="47" t="s">
         <v>263</v>
       </c>
-      <c r="H531" s="117"/>
+      <c r="H531" s="116"/>
     </row>
     <row r="532" spans="1:8">
-      <c r="A532" s="108" t="s">
+      <c r="A532" s="107" t="s">
         <v>547</v>
       </c>
       <c r="B532" s="8" t="s">
@@ -16270,7 +16267,7 @@
       </c>
     </row>
     <row r="534" spans="1:8">
-      <c r="A534" s="96" t="s">
+      <c r="A534" s="95" t="s">
         <v>549</v>
       </c>
       <c r="B534" s="8" t="s">
@@ -16385,7 +16382,7 @@
       </c>
     </row>
     <row r="539" spans="1:8">
-      <c r="A539" s="86" t="s">
+      <c r="A539" s="85" t="s">
         <v>554</v>
       </c>
       <c r="B539" s="8" t="s">
@@ -16408,7 +16405,7 @@
       </c>
     </row>
     <row r="540" spans="1:8">
-      <c r="A540" s="99" t="s">
+      <c r="A540" s="98" t="s">
         <v>555</v>
       </c>
       <c r="B540" s="8" t="s">
@@ -16431,7 +16428,7 @@
       </c>
     </row>
     <row r="541" spans="1:8">
-      <c r="A541" s="79" t="s">
+      <c r="A541" s="78" t="s">
         <v>557</v>
       </c>
       <c r="B541" s="8" t="s">
@@ -16454,7 +16451,7 @@
       </c>
     </row>
     <row r="542" spans="1:8">
-      <c r="A542" s="93" t="s">
+      <c r="A542" s="92" t="s">
         <v>556</v>
       </c>
       <c r="B542" s="8" t="s">
@@ -16477,7 +16474,7 @@
       </c>
     </row>
     <row r="543" spans="1:8">
-      <c r="A543" s="92" t="s">
+      <c r="A543" s="91" t="s">
         <v>558</v>
       </c>
       <c r="B543" s="8" t="s">
@@ -16500,7 +16497,7 @@
       </c>
     </row>
     <row r="544" spans="1:8">
-      <c r="A544" s="72" t="s">
+      <c r="A544" s="71" t="s">
         <v>559</v>
       </c>
       <c r="B544" s="8" t="s">
@@ -16638,7 +16635,7 @@
       </c>
     </row>
     <row r="550" spans="1:7">
-      <c r="A550" s="118" t="s">
+      <c r="A550" s="117" t="s">
         <v>565</v>
       </c>
       <c r="B550" s="8" t="s">
@@ -16661,7 +16658,7 @@
       </c>
     </row>
     <row r="551" spans="1:7">
-      <c r="A551" s="110" t="s">
+      <c r="A551" s="109" t="s">
         <v>566</v>
       </c>
       <c r="B551" s="8" t="s">
@@ -16684,7 +16681,7 @@
       </c>
     </row>
     <row r="552" spans="1:7">
-      <c r="A552" s="98" t="s">
+      <c r="A552" s="97" t="s">
         <v>567</v>
       </c>
       <c r="B552" s="8" t="s">
@@ -16776,7 +16773,7 @@
       </c>
     </row>
     <row r="556" spans="1:7">
-      <c r="A556" s="119" t="s">
+      <c r="A556" s="118" t="s">
         <v>571</v>
       </c>
       <c r="B556" s="8" t="s">
@@ -16822,7 +16819,7 @@
       </c>
     </row>
     <row r="558" spans="1:7">
-      <c r="A558" s="69" t="s">
+      <c r="A558" s="68" t="s">
         <v>573</v>
       </c>
       <c r="B558" s="8" t="s">
@@ -16845,7 +16842,7 @@
       </c>
     </row>
     <row r="559" spans="1:7">
-      <c r="A559" s="79" t="s">
+      <c r="A559" s="78" t="s">
         <v>574</v>
       </c>
       <c r="B559" s="8" t="s">
@@ -16868,7 +16865,7 @@
       </c>
     </row>
     <row r="560" spans="1:7">
-      <c r="A560" s="120" t="s">
+      <c r="A560" s="119" t="s">
         <v>575</v>
       </c>
       <c r="B560" s="8" t="s">
@@ -16891,7 +16888,7 @@
       </c>
     </row>
     <row r="561" spans="1:7">
-      <c r="A561" s="100" t="s">
+      <c r="A561" s="99" t="s">
         <v>576</v>
       </c>
       <c r="B561" s="8" t="s">
@@ -16914,7 +16911,7 @@
       </c>
     </row>
     <row r="562" spans="1:7">
-      <c r="A562" s="99" t="s">
+      <c r="A562" s="98" t="s">
         <v>577</v>
       </c>
       <c r="B562" s="8" t="s">
@@ -16937,7 +16934,7 @@
       </c>
     </row>
     <row r="563" spans="1:7">
-      <c r="A563" s="103" t="s">
+      <c r="A563" s="102" t="s">
         <v>578</v>
       </c>
       <c r="B563" s="8" t="s">
@@ -16960,7 +16957,7 @@
       </c>
     </row>
     <row r="564" spans="1:7">
-      <c r="A564" s="121" t="s">
+      <c r="A564" s="120" t="s">
         <v>579</v>
       </c>
       <c r="B564" s="8" t="s">
@@ -17006,7 +17003,7 @@
       </c>
     </row>
     <row r="566" spans="1:7">
-      <c r="A566" s="87" t="s">
+      <c r="A566" s="86" t="s">
         <v>581</v>
       </c>
       <c r="B566" s="8" t="s">
@@ -17029,7 +17026,7 @@
       </c>
     </row>
     <row r="567" spans="1:7">
-      <c r="A567" s="108" t="s">
+      <c r="A567" s="107" t="s">
         <v>582</v>
       </c>
       <c r="B567" s="8" t="s">
@@ -17075,7 +17072,7 @@
       </c>
     </row>
     <row r="569" spans="1:7">
-      <c r="A569" s="99" t="s">
+      <c r="A569" s="98" t="s">
         <v>584</v>
       </c>
       <c r="B569" s="8" t="s">
@@ -17121,7 +17118,7 @@
       </c>
     </row>
     <row r="571" spans="1:7">
-      <c r="A571" s="121" t="s">
+      <c r="A571" s="120" t="s">
         <v>586</v>
       </c>
       <c r="B571" s="8" t="s">
@@ -17282,7 +17279,7 @@
       </c>
     </row>
     <row r="578" spans="1:7">
-      <c r="A578" s="111" t="s">
+      <c r="A578" s="110" t="s">
         <v>593</v>
       </c>
       <c r="B578" s="8" t="s">
@@ -17305,7 +17302,7 @@
       </c>
     </row>
     <row r="579" spans="1:7">
-      <c r="A579" s="92" t="s">
+      <c r="A579" s="91" t="s">
         <v>594</v>
       </c>
       <c r="B579" s="8" t="s">
@@ -17328,7 +17325,7 @@
       </c>
     </row>
     <row r="580" spans="1:7">
-      <c r="A580" s="93" t="s">
+      <c r="A580" s="92" t="s">
         <v>595</v>
       </c>
       <c r="B580" s="8" t="s">
@@ -17397,7 +17394,7 @@
       </c>
     </row>
     <row r="583" spans="1:7">
-      <c r="A583" s="71" t="s">
+      <c r="A583" s="70" t="s">
         <v>598</v>
       </c>
       <c r="B583" s="8" t="s">
@@ -17466,7 +17463,7 @@
       </c>
     </row>
     <row r="586" spans="1:7">
-      <c r="A586" s="111" t="s">
+      <c r="A586" s="110" t="s">
         <v>600</v>
       </c>
       <c r="B586" s="8" t="s">
@@ -17489,7 +17486,7 @@
       </c>
     </row>
     <row r="587" spans="1:7">
-      <c r="A587" s="122" t="s">
+      <c r="A587" s="121" t="s">
         <v>601</v>
       </c>
       <c r="B587" s="8" t="s">
@@ -17535,7 +17532,7 @@
       </c>
     </row>
     <row r="589" spans="1:7">
-      <c r="A589" s="123" t="s">
+      <c r="A589" s="122" t="s">
         <v>603</v>
       </c>
       <c r="B589" s="8" t="s">
@@ -17558,7 +17555,7 @@
       </c>
     </row>
     <row r="590" spans="1:7">
-      <c r="A590" s="121" t="s">
+      <c r="A590" s="120" t="s">
         <v>604</v>
       </c>
       <c r="B590" s="8" t="s">
@@ -17581,7 +17578,7 @@
       </c>
     </row>
     <row r="591" spans="1:7">
-      <c r="A591" s="98" t="s">
+      <c r="A591" s="97" t="s">
         <v>605</v>
       </c>
       <c r="B591" s="8" t="s">
@@ -17604,7 +17601,7 @@
       </c>
     </row>
     <row r="592" spans="1:7">
-      <c r="A592" s="124" t="s">
+      <c r="A592" s="123" t="s">
         <v>606</v>
       </c>
       <c r="B592" s="8" t="s">
@@ -17627,7 +17624,7 @@
       </c>
     </row>
     <row r="593" spans="1:7">
-      <c r="A593" s="102" t="s">
+      <c r="A593" s="101" t="s">
         <v>607</v>
       </c>
       <c r="B593" s="8" t="s">
@@ -17650,7 +17647,7 @@
       </c>
     </row>
     <row r="594" spans="1:7">
-      <c r="A594" s="125" t="s">
+      <c r="A594" s="124" t="s">
         <v>608</v>
       </c>
       <c r="B594" s="8" t="s">
@@ -17673,7 +17670,7 @@
       </c>
     </row>
     <row r="595" spans="1:7">
-      <c r="A595" s="107" t="s">
+      <c r="A595" s="106" t="s">
         <v>609</v>
       </c>
       <c r="B595" s="8" t="s">
@@ -17696,7 +17693,7 @@
       </c>
     </row>
     <row r="596" spans="1:7">
-      <c r="A596" s="73" t="s">
+      <c r="A596" s="72" t="s">
         <v>610</v>
       </c>
       <c r="B596" s="8" t="s">
@@ -17719,7 +17716,7 @@
       </c>
     </row>
     <row r="597" spans="1:7">
-      <c r="A597" s="126" t="s">
+      <c r="A597" s="125" t="s">
         <v>611</v>
       </c>
       <c r="B597" s="8" t="s">
@@ -17742,7 +17739,7 @@
       </c>
     </row>
     <row r="598" spans="1:7">
-      <c r="A598" s="78" t="s">
+      <c r="A598" s="77" t="s">
         <v>612</v>
       </c>
       <c r="B598" s="8" t="s">
@@ -17811,7 +17808,7 @@
       </c>
     </row>
     <row r="601" spans="1:7">
-      <c r="A601" s="106" t="s">
+      <c r="A601" s="105" t="s">
         <v>615</v>
       </c>
       <c r="B601" s="8" t="s">
@@ -17834,7 +17831,7 @@
       </c>
     </row>
     <row r="602" spans="1:7">
-      <c r="A602" s="126" t="s">
+      <c r="A602" s="125" t="s">
         <v>617</v>
       </c>
       <c r="B602" s="8" t="s">
@@ -17857,7 +17854,7 @@
       </c>
     </row>
     <row r="603" spans="1:7">
-      <c r="A603" s="124" t="s">
+      <c r="A603" s="123" t="s">
         <v>616</v>
       </c>
       <c r="B603" s="8" t="s">
@@ -17880,7 +17877,7 @@
       </c>
     </row>
     <row r="604" spans="1:7">
-      <c r="A604" s="72" t="s">
+      <c r="A604" s="71" t="s">
         <v>618</v>
       </c>
       <c r="B604" s="8" t="s">
@@ -17903,7 +17900,7 @@
       </c>
     </row>
     <row r="605" spans="1:7">
-      <c r="A605" s="75" t="s">
+      <c r="A605" s="74" t="s">
         <v>619</v>
       </c>
       <c r="B605" s="8" t="s">
@@ -17926,7 +17923,7 @@
       </c>
     </row>
     <row r="606" spans="1:7">
-      <c r="A606" s="106" t="s">
+      <c r="A606" s="105" t="s">
         <v>620</v>
       </c>
       <c r="B606" s="8" t="s">
@@ -17949,7 +17946,7 @@
       </c>
     </row>
     <row r="607" spans="1:7">
-      <c r="A607" s="108" t="s">
+      <c r="A607" s="107" t="s">
         <v>621</v>
       </c>
       <c r="B607" s="8" t="s">
@@ -17972,7 +17969,7 @@
       </c>
     </row>
     <row r="608" spans="1:7">
-      <c r="A608" s="102" t="s">
+      <c r="A608" s="101" t="s">
         <v>622</v>
       </c>
       <c r="B608" s="8" t="s">
@@ -17995,7 +17992,7 @@
       </c>
     </row>
     <row r="609" spans="1:7">
-      <c r="A609" s="88" t="s">
+      <c r="A609" s="87" t="s">
         <v>623</v>
       </c>
       <c r="B609" s="8" t="s">
@@ -18018,7 +18015,7 @@
       </c>
     </row>
     <row r="610" spans="1:7">
-      <c r="A610" s="127" t="s">
+      <c r="A610" s="126" t="s">
         <v>624</v>
       </c>
       <c r="B610" s="8" t="s">
@@ -18041,7 +18038,7 @@
       </c>
     </row>
     <row r="611" spans="1:7">
-      <c r="A611" s="122" t="s">
+      <c r="A611" s="121" t="s">
         <v>625</v>
       </c>
       <c r="B611" s="8" t="s">
@@ -18087,7 +18084,7 @@
       </c>
     </row>
     <row r="613" spans="1:7">
-      <c r="A613" s="121" t="s">
+      <c r="A613" s="120" t="s">
         <v>627</v>
       </c>
       <c r="B613" s="8" t="s">
@@ -18110,7 +18107,7 @@
       </c>
     </row>
     <row r="614" spans="1:7">
-      <c r="A614" s="93" t="s">
+      <c r="A614" s="92" t="s">
         <v>628</v>
       </c>
       <c r="B614" s="8" t="s">
@@ -18133,7 +18130,7 @@
       </c>
     </row>
     <row r="615" spans="1:7">
-      <c r="A615" s="75" t="s">
+      <c r="A615" s="74" t="s">
         <v>629</v>
       </c>
       <c r="B615" s="8" t="s">
@@ -18156,7 +18153,7 @@
       </c>
     </row>
     <row r="616" spans="1:7">
-      <c r="A616" s="124" t="s">
+      <c r="A616" s="123" t="s">
         <v>630</v>
       </c>
       <c r="B616" s="8" t="s">
@@ -18179,7 +18176,7 @@
       </c>
     </row>
     <row r="617" spans="1:7">
-      <c r="A617" s="86" t="s">
+      <c r="A617" s="85" t="s">
         <v>631</v>
       </c>
       <c r="B617" s="8" t="s">
@@ -18202,7 +18199,7 @@
       </c>
     </row>
     <row r="618" spans="1:7">
-      <c r="A618" s="110" t="s">
+      <c r="A618" s="109" t="s">
         <v>632</v>
       </c>
       <c r="B618" s="8" t="s">
@@ -18225,7 +18222,7 @@
       </c>
     </row>
     <row r="619" spans="1:7">
-      <c r="A619" s="78" t="s">
+      <c r="A619" s="77" t="s">
         <v>633</v>
       </c>
       <c r="B619" s="8" t="s">
@@ -18248,7 +18245,7 @@
       </c>
     </row>
     <row r="620" spans="1:7">
-      <c r="A620" s="98" t="s">
+      <c r="A620" s="97" t="s">
         <v>634</v>
       </c>
       <c r="B620" s="8" t="s">
@@ -18271,7 +18268,7 @@
       </c>
     </row>
     <row r="621" spans="1:7">
-      <c r="A621" s="77" t="s">
+      <c r="A621" s="76" t="s">
         <v>635</v>
       </c>
       <c r="B621" s="8" t="s">
@@ -18294,7 +18291,7 @@
       </c>
     </row>
     <row r="622" spans="1:7">
-      <c r="A622" s="107" t="s">
+      <c r="A622" s="106" t="s">
         <v>636</v>
       </c>
       <c r="B622" s="8" t="s">
@@ -18340,7 +18337,7 @@
       </c>
     </row>
     <row r="624" spans="1:7">
-      <c r="A624" s="102" t="s">
+      <c r="A624" s="101" t="s">
         <v>637</v>
       </c>
       <c r="B624" s="8" t="s">
@@ -18363,7 +18360,7 @@
       </c>
     </row>
     <row r="625" spans="1:7">
-      <c r="A625" s="67" t="s">
+      <c r="A625" s="66" t="s">
         <v>638</v>
       </c>
       <c r="B625" s="8" t="s">
@@ -18386,7 +18383,7 @@
       </c>
     </row>
     <row r="626" spans="1:7">
-      <c r="A626" s="128" t="s">
+      <c r="A626" s="127" t="s">
         <v>639</v>
       </c>
       <c r="B626" s="8" t="s">
@@ -18409,7 +18406,7 @@
       </c>
     </row>
     <row r="627" spans="1:7">
-      <c r="A627" s="109" t="s">
+      <c r="A627" s="108" t="s">
         <v>640</v>
       </c>
       <c r="B627" s="8" t="s">
@@ -18432,7 +18429,7 @@
       </c>
     </row>
     <row r="628" spans="1:7">
-      <c r="A628" s="123" t="s">
+      <c r="A628" s="122" t="s">
         <v>641</v>
       </c>
       <c r="B628" s="8" t="s">
@@ -18478,7 +18475,7 @@
       </c>
     </row>
     <row r="630" spans="1:7">
-      <c r="A630" s="129" t="s">
+      <c r="A630" s="128" t="s">
         <v>643</v>
       </c>
       <c r="B630" s="8" t="s">
@@ -18524,7 +18521,7 @@
       </c>
     </row>
     <row r="632" spans="1:7">
-      <c r="A632" s="130" t="s">
+      <c r="A632" s="129" t="s">
         <v>646</v>
       </c>
       <c r="B632" s="8" t="s">
@@ -18593,7 +18590,7 @@
       </c>
     </row>
     <row r="635" spans="1:7">
-      <c r="A635" s="131" t="s">
+      <c r="A635" s="130" t="s">
         <v>649</v>
       </c>
       <c r="B635" s="8" t="s">
@@ -18616,7 +18613,7 @@
       </c>
     </row>
     <row r="636" spans="1:7">
-      <c r="A636" s="132" t="s">
+      <c r="A636" s="131" t="s">
         <v>651</v>
       </c>
       <c r="B636" s="8" t="s">
@@ -18639,7 +18636,7 @@
       </c>
     </row>
     <row r="637" spans="1:7">
-      <c r="A637" s="119" t="s">
+      <c r="A637" s="118" t="s">
         <v>652</v>
       </c>
       <c r="B637" s="8" t="s">
@@ -18662,7 +18659,7 @@
       </c>
     </row>
     <row r="638" spans="1:7">
-      <c r="A638" s="133" t="s">
+      <c r="A638" s="132" t="s">
         <v>653</v>
       </c>
       <c r="B638" s="8" t="s">
@@ -18685,7 +18682,7 @@
       </c>
     </row>
     <row r="639" spans="1:7">
-      <c r="A639" s="105" t="s">
+      <c r="A639" s="104" t="s">
         <v>654</v>
       </c>
       <c r="B639" s="8" t="s">
@@ -18731,7 +18728,7 @@
       </c>
     </row>
     <row r="641" spans="1:7">
-      <c r="A641" s="120" t="s">
+      <c r="A641" s="119" t="s">
         <v>656</v>
       </c>
       <c r="B641" s="8" t="s">
@@ -18754,7 +18751,7 @@
       </c>
     </row>
     <row r="642" spans="1:7">
-      <c r="A642" s="93" t="s">
+      <c r="A642" s="92" t="s">
         <v>658</v>
       </c>
       <c r="B642" s="8" t="s">
@@ -18777,7 +18774,7 @@
       </c>
     </row>
     <row r="643" spans="1:7">
-      <c r="A643" s="126" t="s">
+      <c r="A643" s="125" t="s">
         <v>659</v>
       </c>
       <c r="B643" s="8" t="s">
@@ -18800,7 +18797,7 @@
       </c>
     </row>
     <row r="644" spans="1:7">
-      <c r="A644" s="134" t="s">
+      <c r="A644" s="133" t="s">
         <v>660</v>
       </c>
       <c r="B644" s="8" t="s">
@@ -18823,7 +18820,7 @@
       </c>
     </row>
     <row r="645" spans="1:7">
-      <c r="A645" s="99" t="s">
+      <c r="A645" s="98" t="s">
         <v>661</v>
       </c>
       <c r="B645" s="8" t="s">
@@ -18869,7 +18866,7 @@
       </c>
     </row>
     <row r="647" spans="1:7">
-      <c r="A647" s="126" t="s">
+      <c r="A647" s="125" t="s">
         <v>663</v>
       </c>
       <c r="B647" s="8" t="s">
@@ -18892,7 +18889,7 @@
       </c>
     </row>
     <row r="648" spans="1:7">
-      <c r="A648" s="108" t="s">
+      <c r="A648" s="107" t="s">
         <v>664</v>
       </c>
       <c r="B648" s="8" t="s">
@@ -18915,7 +18912,7 @@
       </c>
     </row>
     <row r="649" spans="1:7">
-      <c r="A649" s="67" t="s">
+      <c r="A649" s="66" t="s">
         <v>665</v>
       </c>
       <c r="B649" s="8" t="s">
@@ -18984,7 +18981,7 @@
       </c>
     </row>
     <row r="652" spans="1:7">
-      <c r="A652" s="85" t="s">
+      <c r="A652" s="84" t="s">
         <v>668</v>
       </c>
       <c r="B652" s="8" t="s">
@@ -19007,7 +19004,7 @@
       </c>
     </row>
     <row r="653" spans="1:7">
-      <c r="A653" s="122" t="s">
+      <c r="A653" s="121" t="s">
         <v>669</v>
       </c>
       <c r="B653" s="8" t="s">
@@ -19030,7 +19027,7 @@
       </c>
     </row>
     <row r="654" spans="1:7">
-      <c r="A654" s="72" t="s">
+      <c r="A654" s="71" t="s">
         <v>670</v>
       </c>
       <c r="B654" s="8" t="s">
@@ -19053,7 +19050,7 @@
       </c>
     </row>
     <row r="655" spans="1:7">
-      <c r="A655" s="93" t="s">
+      <c r="A655" s="92" t="s">
         <v>671</v>
       </c>
       <c r="B655" s="8" t="s">
@@ -19099,7 +19096,7 @@
       </c>
     </row>
     <row r="657" spans="1:8">
-      <c r="A657" s="75" t="s">
+      <c r="A657" s="74" t="s">
         <v>673</v>
       </c>
       <c r="B657" s="8" t="s">
@@ -19122,7 +19119,7 @@
       </c>
     </row>
     <row r="658" spans="1:8">
-      <c r="A658" s="92" t="s">
+      <c r="A658" s="91" t="s">
         <v>674</v>
       </c>
       <c r="B658" s="8" t="s">
@@ -19145,7 +19142,7 @@
       </c>
     </row>
     <row r="659" spans="1:8">
-      <c r="A659" s="81" t="s">
+      <c r="A659" s="80" t="s">
         <v>675</v>
       </c>
       <c r="B659" s="8" t="s">
@@ -19166,12 +19163,12 @@
       <c r="G659" s="34" t="s">
         <v>263</v>
       </c>
-      <c r="H659" s="117" t="s">
+      <c r="H659" s="116" t="s">
         <v>650</v>
       </c>
     </row>
     <row r="660" spans="1:8">
-      <c r="A660" s="135" t="s">
+      <c r="A660" s="134" t="s">
         <v>676</v>
       </c>
       <c r="B660" s="8" t="s">
@@ -19194,7 +19191,7 @@
       </c>
     </row>
     <row r="661" spans="1:8">
-      <c r="A661" s="67" t="s">
+      <c r="A661" s="66" t="s">
         <v>677</v>
       </c>
       <c r="B661" s="8" t="s">
@@ -19217,7 +19214,7 @@
       </c>
     </row>
     <row r="662" spans="1:8">
-      <c r="A662" s="101" t="s">
+      <c r="A662" s="100" t="s">
         <v>678</v>
       </c>
       <c r="B662" s="8" t="s">
@@ -19240,7 +19237,7 @@
       </c>
     </row>
     <row r="663" spans="1:8">
-      <c r="A663" s="122" t="s">
+      <c r="A663" s="121" t="s">
         <v>679</v>
       </c>
       <c r="B663" s="8" t="s">
@@ -19263,7 +19260,7 @@
       </c>
     </row>
     <row r="664" spans="1:8">
-      <c r="A664" s="136" t="s">
+      <c r="A664" s="135" t="s">
         <v>680</v>
       </c>
       <c r="B664" s="8" t="s">
@@ -19286,7 +19283,7 @@
       </c>
     </row>
     <row r="665" spans="1:8">
-      <c r="A665" s="98" t="s">
+      <c r="A665" s="97" t="s">
         <v>681</v>
       </c>
       <c r="B665" s="8" t="s">
@@ -19309,7 +19306,7 @@
       </c>
     </row>
     <row r="666" spans="1:8">
-      <c r="A666" s="109" t="s">
+      <c r="A666" s="108" t="s">
         <v>744</v>
       </c>
       <c r="B666" s="8" t="s">
@@ -19332,7 +19329,7 @@
       </c>
     </row>
     <row r="667" spans="1:8">
-      <c r="A667" s="75" t="s">
+      <c r="A667" s="74" t="s">
         <v>682</v>
       </c>
       <c r="B667" s="8" t="s">
@@ -19355,7 +19352,7 @@
       </c>
     </row>
     <row r="668" spans="1:8">
-      <c r="A668" s="121" t="s">
+      <c r="A668" s="120" t="s">
         <v>683</v>
       </c>
       <c r="B668" s="8" t="s">
@@ -19378,7 +19375,7 @@
       </c>
     </row>
     <row r="669" spans="1:8">
-      <c r="A669" s="86" t="s">
+      <c r="A669" s="85" t="s">
         <v>684</v>
       </c>
       <c r="B669" s="8" t="s">
@@ -19424,7 +19421,7 @@
       </c>
     </row>
     <row r="671" spans="1:8">
-      <c r="A671" s="137" t="s">
+      <c r="A671" s="136" t="s">
         <v>686</v>
       </c>
       <c r="B671" s="8" t="s">
@@ -19447,7 +19444,7 @@
       </c>
     </row>
     <row r="672" spans="1:8">
-      <c r="A672" s="80" t="s">
+      <c r="A672" s="79" t="s">
         <v>687</v>
       </c>
       <c r="B672" s="8" t="s">
@@ -19470,7 +19467,7 @@
       </c>
     </row>
     <row r="673" spans="1:7">
-      <c r="A673" s="109" t="s">
+      <c r="A673" s="108" t="s">
         <v>688</v>
       </c>
       <c r="B673" s="8" t="s">
@@ -19493,7 +19490,7 @@
       </c>
     </row>
     <row r="674" spans="1:7">
-      <c r="A674" s="120" t="s">
+      <c r="A674" s="119" t="s">
         <v>689</v>
       </c>
       <c r="B674" s="8" t="s">
@@ -19516,7 +19513,7 @@
       </c>
     </row>
     <row r="675" spans="1:7">
-      <c r="A675" s="108" t="s">
+      <c r="A675" s="107" t="s">
         <v>690</v>
       </c>
       <c r="B675" s="8" t="s">
@@ -19539,7 +19536,7 @@
       </c>
     </row>
     <row r="676" spans="1:7">
-      <c r="A676" s="122" t="s">
+      <c r="A676" s="121" t="s">
         <v>691</v>
       </c>
       <c r="B676" s="8" t="s">
@@ -19562,7 +19559,7 @@
       </c>
     </row>
     <row r="677" spans="1:7">
-      <c r="A677" s="106" t="s">
+      <c r="A677" s="105" t="s">
         <v>692</v>
       </c>
       <c r="B677" s="8" t="s">
@@ -19585,7 +19582,7 @@
       </c>
     </row>
     <row r="678" spans="1:7" ht="16.5">
-      <c r="A678" s="138" t="s">
+      <c r="A678" s="137" t="s">
         <v>693</v>
       </c>
       <c r="B678" s="8" t="s">
@@ -19608,7 +19605,7 @@
       </c>
     </row>
     <row r="679" spans="1:7">
-      <c r="A679" s="101" t="s">
+      <c r="A679" s="100" t="s">
         <v>694</v>
       </c>
       <c r="B679" s="8" t="s">
@@ -19631,7 +19628,7 @@
       </c>
     </row>
     <row r="680" spans="1:7">
-      <c r="A680" s="139" t="s">
+      <c r="A680" s="138" t="s">
         <v>695</v>
       </c>
       <c r="B680" s="8" t="s">
@@ -19654,7 +19651,7 @@
       </c>
     </row>
     <row r="681" spans="1:7">
-      <c r="A681" s="85" t="s">
+      <c r="A681" s="84" t="s">
         <v>696</v>
       </c>
       <c r="B681" s="8" t="s">
@@ -19700,7 +19697,7 @@
       </c>
     </row>
     <row r="683" spans="1:7">
-      <c r="A683" s="140" t="s">
+      <c r="A683" s="139" t="s">
         <v>698</v>
       </c>
       <c r="B683" s="8" t="s">
@@ -19723,7 +19720,7 @@
       </c>
     </row>
     <row r="684" spans="1:7" ht="16.5">
-      <c r="A684" s="141" t="s">
+      <c r="A684" s="140" t="s">
         <v>699</v>
       </c>
       <c r="B684" s="8" t="s">
@@ -19746,7 +19743,7 @@
       </c>
     </row>
     <row r="685" spans="1:7" ht="16.5">
-      <c r="A685" s="142" t="s">
+      <c r="A685" s="141" t="s">
         <v>700</v>
       </c>
       <c r="B685" s="8" t="s">
@@ -19769,7 +19766,7 @@
       </c>
     </row>
     <row r="686" spans="1:7">
-      <c r="A686" s="110" t="s">
+      <c r="A686" s="109" t="s">
         <v>701</v>
       </c>
       <c r="B686" s="8" t="s">
@@ -19792,7 +19789,7 @@
       </c>
     </row>
     <row r="687" spans="1:7">
-      <c r="A687" s="90" t="s">
+      <c r="A687" s="89" t="s">
         <v>702</v>
       </c>
       <c r="B687" s="8" t="s">
@@ -19815,7 +19812,7 @@
       </c>
     </row>
     <row r="688" spans="1:7">
-      <c r="A688" s="75" t="s">
+      <c r="A688" s="74" t="s">
         <v>703</v>
       </c>
       <c r="B688" s="8" t="s">
@@ -19838,7 +19835,7 @@
       </c>
     </row>
     <row r="689" spans="1:7">
-      <c r="A689" s="101" t="s">
+      <c r="A689" s="100" t="s">
         <v>704</v>
       </c>
       <c r="B689" s="8" t="s">
@@ -19861,7 +19858,7 @@
       </c>
     </row>
     <row r="690" spans="1:7" ht="16.5">
-      <c r="A690" s="143" t="s">
+      <c r="A690" s="142" t="s">
         <v>705</v>
       </c>
       <c r="B690" s="8" t="s">
@@ -19930,7 +19927,7 @@
       </c>
     </row>
     <row r="693" spans="1:7">
-      <c r="A693" s="109" t="s">
+      <c r="A693" s="108" t="s">
         <v>708</v>
       </c>
       <c r="B693" s="8" t="s">
@@ -19976,7 +19973,7 @@
       </c>
     </row>
     <row r="695" spans="1:7">
-      <c r="A695" s="69" t="s">
+      <c r="A695" s="68" t="s">
         <v>710</v>
       </c>
       <c r="B695" s="8" t="s">
@@ -19999,7 +19996,7 @@
       </c>
     </row>
     <row r="696" spans="1:7">
-      <c r="A696" s="122" t="s">
+      <c r="A696" s="121" t="s">
         <v>711</v>
       </c>
       <c r="B696" s="8" t="s">
@@ -20045,7 +20042,7 @@
       </c>
     </row>
     <row r="698" spans="1:7">
-      <c r="A698" s="82" t="s">
+      <c r="A698" s="81" t="s">
         <v>713</v>
       </c>
       <c r="B698" s="8" t="s">
@@ -20114,7 +20111,7 @@
       </c>
     </row>
     <row r="701" spans="1:7">
-      <c r="A701" s="122" t="s">
+      <c r="A701" s="121" t="s">
         <v>716</v>
       </c>
       <c r="B701" s="8" t="s">
@@ -20160,7 +20157,7 @@
       </c>
     </row>
     <row r="703" spans="1:7">
-      <c r="A703" s="103" t="s">
+      <c r="A703" s="102" t="s">
         <v>718</v>
       </c>
       <c r="B703" s="8" t="s">
@@ -20206,7 +20203,7 @@
       </c>
     </row>
     <row r="705" spans="1:7">
-      <c r="A705" s="111" t="s">
+      <c r="A705" s="110" t="s">
         <v>720</v>
       </c>
       <c r="B705" s="8" t="s">
@@ -20275,7 +20272,7 @@
       </c>
     </row>
     <row r="708" spans="1:7">
-      <c r="A708" s="135" t="s">
+      <c r="A708" s="134" t="s">
         <v>723</v>
       </c>
       <c r="B708" s="8" t="s">
@@ -20344,7 +20341,7 @@
       </c>
     </row>
     <row r="711" spans="1:7">
-      <c r="A711" s="73" t="s">
+      <c r="A711" s="72" t="s">
         <v>732</v>
       </c>
       <c r="B711" s="8" t="s">
@@ -20367,7 +20364,7 @@
       </c>
     </row>
     <row r="712" spans="1:7">
-      <c r="A712" s="91" t="s">
+      <c r="A712" s="90" t="s">
         <v>733</v>
       </c>
       <c r="B712" s="8" t="s">
@@ -20390,7 +20387,7 @@
       </c>
     </row>
     <row r="713" spans="1:7">
-      <c r="A713" s="69" t="s">
+      <c r="A713" s="68" t="s">
         <v>740</v>
       </c>
       <c r="B713" s="8" t="s">
@@ -20413,7 +20410,7 @@
       </c>
     </row>
     <row r="714" spans="1:7">
-      <c r="A714" s="67" t="s">
+      <c r="A714" s="66" t="s">
         <v>741</v>
       </c>
       <c r="B714" s="8" t="s">
@@ -20459,7 +20456,7 @@
       </c>
     </row>
     <row r="716" spans="1:7">
-      <c r="A716" s="75" t="s">
+      <c r="A716" s="74" t="s">
         <v>746</v>
       </c>
       <c r="B716" s="8" t="s">
@@ -20505,7 +20502,7 @@
       </c>
     </row>
     <row r="718" spans="1:7">
-      <c r="A718" s="106" t="s">
+      <c r="A718" s="105" t="s">
         <v>748</v>
       </c>
       <c r="B718" s="8" t="s">
@@ -20528,7 +20525,7 @@
       </c>
     </row>
     <row r="719" spans="1:7">
-      <c r="A719" s="67" t="s">
+      <c r="A719" s="66" t="s">
         <v>749</v>
       </c>
       <c r="B719" s="8" t="s">
@@ -20574,7 +20571,7 @@
       </c>
     </row>
     <row r="721" spans="1:7">
-      <c r="A721" s="140" t="s">
+      <c r="A721" s="139" t="s">
         <v>751</v>
       </c>
       <c r="B721" s="8" t="s">
@@ -20597,7 +20594,7 @@
       </c>
     </row>
     <row r="722" spans="1:7">
-      <c r="A722" s="144" t="s">
+      <c r="A722" s="143" t="s">
         <v>752</v>
       </c>
       <c r="B722" s="8" t="s">
@@ -20666,7 +20663,7 @@
       </c>
     </row>
     <row r="725" spans="1:7">
-      <c r="A725" s="101" t="s">
+      <c r="A725" s="100" t="s">
         <v>755</v>
       </c>
       <c r="B725" s="8" t="s">
@@ -20689,7 +20686,7 @@
       </c>
     </row>
     <row r="726" spans="1:7">
-      <c r="A726" s="88" t="s">
+      <c r="A726" s="87" t="s">
         <v>756</v>
       </c>
       <c r="B726" s="8" t="s">
@@ -20712,7 +20709,7 @@
       </c>
     </row>
     <row r="727" spans="1:7">
-      <c r="A727" s="139" t="s">
+      <c r="A727" s="138" t="s">
         <v>757</v>
       </c>
       <c r="B727" s="8" t="s">
@@ -20735,7 +20732,7 @@
       </c>
     </row>
     <row r="728" spans="1:7">
-      <c r="A728" s="85" t="s">
+      <c r="A728" s="84" t="s">
         <v>758</v>
       </c>
       <c r="B728" s="8" t="s">
@@ -20758,7 +20755,7 @@
       </c>
     </row>
     <row r="729" spans="1:7">
-      <c r="A729" s="86" t="s">
+      <c r="A729" s="85" t="s">
         <v>759</v>
       </c>
       <c r="B729" s="8" t="s">
@@ -20781,7 +20778,7 @@
       </c>
     </row>
     <row r="730" spans="1:7">
-      <c r="A730" s="103" t="s">
+      <c r="A730" s="102" t="s">
         <v>760</v>
       </c>
       <c r="B730" s="8" t="s">
@@ -20804,7 +20801,7 @@
       </c>
     </row>
     <row r="731" spans="1:7">
-      <c r="A731" s="96" t="s">
+      <c r="A731" s="95" t="s">
         <v>761</v>
       </c>
       <c r="B731" s="8" t="s">
@@ -20827,7 +20824,7 @@
       </c>
     </row>
     <row r="732" spans="1:7">
-      <c r="A732" s="135" t="s">
+      <c r="A732" s="134" t="s">
         <v>762</v>
       </c>
       <c r="B732" s="8" t="s">
@@ -20850,7 +20847,7 @@
       </c>
     </row>
     <row r="733" spans="1:7">
-      <c r="A733" s="139" t="s">
+      <c r="A733" s="138" t="s">
         <v>763</v>
       </c>
       <c r="B733" s="8" t="s">
@@ -20873,7 +20870,7 @@
       </c>
     </row>
     <row r="734" spans="1:7">
-      <c r="A734" s="99" t="s">
+      <c r="A734" s="98" t="s">
         <v>764</v>
       </c>
       <c r="B734" s="8" t="s">
@@ -20896,7 +20893,7 @@
       </c>
     </row>
     <row r="735" spans="1:7">
-      <c r="A735" s="103" t="s">
+      <c r="A735" s="102" t="s">
         <v>765</v>
       </c>
       <c r="B735" s="8" t="s">
@@ -20942,7 +20939,7 @@
       </c>
     </row>
     <row r="737" spans="1:7">
-      <c r="A737" s="71" t="s">
+      <c r="A737" s="70" t="s">
         <v>767</v>
       </c>
       <c r="B737" s="8" t="s">
@@ -20965,7 +20962,7 @@
       </c>
     </row>
     <row r="738" spans="1:7">
-      <c r="A738" s="145" t="s">
+      <c r="A738" s="144" t="s">
         <v>768</v>
       </c>
       <c r="B738" s="8" t="s">
@@ -20988,7 +20985,7 @@
       </c>
     </row>
     <row r="739" spans="1:7">
-      <c r="A739" s="79" t="s">
+      <c r="A739" s="78" t="s">
         <v>769</v>
       </c>
       <c r="B739" s="8" t="s">
@@ -21011,7 +21008,7 @@
       </c>
     </row>
     <row r="740" spans="1:7">
-      <c r="A740" s="139" t="s">
+      <c r="A740" s="138" t="s">
         <v>770</v>
       </c>
       <c r="B740" s="8" t="s">
@@ -21057,7 +21054,7 @@
       </c>
     </row>
     <row r="742" spans="1:7">
-      <c r="A742" s="70" t="s">
+      <c r="A742" s="69" t="s">
         <v>772</v>
       </c>
       <c r="B742" s="8" t="s">
@@ -21149,7 +21146,7 @@
       </c>
     </row>
     <row r="746" spans="1:7">
-      <c r="A746" s="75" t="s">
+      <c r="A746" s="74" t="s">
         <v>776</v>
       </c>
       <c r="B746" s="8" t="s">
@@ -21172,7 +21169,7 @@
       </c>
     </row>
     <row r="747" spans="1:7">
-      <c r="A747" s="77" t="s">
+      <c r="A747" s="76" t="s">
         <v>777</v>
       </c>
       <c r="B747" s="8" t="s">
@@ -21195,7 +21192,7 @@
       </c>
     </row>
     <row r="748" spans="1:7">
-      <c r="A748" s="88" t="s">
+      <c r="A748" s="87" t="s">
         <v>778</v>
       </c>
       <c r="B748" s="8" t="s">
@@ -21241,7 +21238,7 @@
       </c>
     </row>
     <row r="750" spans="1:7">
-      <c r="A750" s="70" t="s">
+      <c r="A750" s="69" t="s">
         <v>780</v>
       </c>
       <c r="B750" s="8" t="s">
@@ -21264,7 +21261,7 @@
       </c>
     </row>
     <row r="751" spans="1:7">
-      <c r="A751" s="79" t="s">
+      <c r="A751" s="78" t="s">
         <v>781</v>
       </c>
       <c r="B751" s="8" t="s">
@@ -21287,42 +21284,42 @@
       </c>
     </row>
     <row r="752" spans="1:7">
-      <c r="A752" s="139"/>
+      <c r="A752" s="138"/>
     </row>
     <row r="753" spans="1:1">
-      <c r="A753" s="139"/>
+      <c r="A753" s="138"/>
     </row>
     <row r="754" spans="1:1">
-      <c r="A754" s="139"/>
+      <c r="A754" s="138"/>
     </row>
     <row r="755" spans="1:1">
-      <c r="A755" s="139"/>
+      <c r="A755" s="138"/>
     </row>
     <row r="756" spans="1:1">
-      <c r="A756" s="146"/>
+      <c r="A756" s="145"/>
     </row>
     <row r="757" spans="1:1" ht="18.5">
-      <c r="A757" s="150" t="s">
+      <c r="A757" s="149" t="s">
         <v>782</v>
       </c>
     </row>
     <row r="758" spans="1:1" ht="18.5">
-      <c r="A758" s="150" t="s">
+      <c r="A758" s="149" t="s">
         <v>783</v>
       </c>
     </row>
     <row r="759" spans="1:1" ht="18.5">
-      <c r="A759" s="150" t="s">
+      <c r="A759" s="149" t="s">
         <v>787</v>
       </c>
     </row>
     <row r="760" spans="1:1">
-      <c r="A760" s="151" t="s">
+      <c r="A760" s="150" t="s">
         <v>784</v>
       </c>
     </row>
     <row r="779" spans="1:6" ht="15.5">
-      <c r="A779" s="147"/>
+      <c r="A779" s="146"/>
       <c r="B779" s="8"/>
       <c r="C779" s="40"/>
       <c r="D779" s="51"/>
@@ -21330,7 +21327,7 @@
       <c r="F779" s="8"/>
     </row>
     <row r="780" spans="1:6" ht="15.5">
-      <c r="A780" s="147"/>
+      <c r="A780" s="146"/>
       <c r="B780" s="8"/>
       <c r="C780" s="40"/>
       <c r="D780" s="51"/>
@@ -21338,7 +21335,7 @@
       <c r="F780" s="8"/>
     </row>
     <row r="781" spans="1:6" ht="15.5">
-      <c r="A781" s="147"/>
+      <c r="A781" s="146"/>
       <c r="B781" s="8"/>
       <c r="C781" s="40"/>
       <c r="D781" s="51"/>
@@ -21346,7 +21343,7 @@
       <c r="F781" s="8"/>
     </row>
     <row r="782" spans="1:6" ht="15.5">
-      <c r="A782" s="147"/>
+      <c r="A782" s="146"/>
       <c r="B782" s="8"/>
       <c r="C782" s="40"/>
       <c r="D782" s="51"/>

</xml_diff>

<commit_message>
Review 5 Problems 4/23/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57382A24-AA65-46DB-B0B3-2C8D794C8AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC7BF9BC-8222-4417-9CAB-5700DE41A8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2547,7 +2547,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="72">
+  <fonts count="73">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3177,6 +3177,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -3703,10 +3709,10 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFAD8043"/>
       <color rgb="FF308729"/>
       <color rgb="FF800000"/>
       <color rgb="FFEF89E8"/>
-      <color rgb="FFAD8043"/>
       <color rgb="FFB97EFA"/>
       <color rgb="FFEAF4EA"/>
       <color rgb="FFE1E0FE"/>
@@ -9288,7 +9294,7 @@
       <c r="F230" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G230" s="47" t="s">
+      <c r="G230" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9311,7 +9317,7 @@
       <c r="F231" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G231" s="47" t="s">
+      <c r="G231" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9334,7 +9340,7 @@
       <c r="F232" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G232" s="47" t="s">
+      <c r="G232" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9357,7 +9363,7 @@
       <c r="F233" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G233" s="47" t="s">
+      <c r="G233" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9380,7 +9386,7 @@
       <c r="F234" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G234" s="47" t="s">
+      <c r="G234" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -21351,6 +21357,7 @@
       <c r="F782" s="8"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="72" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A484" r:id="rId1" display="https://www.codewars.com/kata/57b68bc7b69bfc8209000307" xr:uid="{B3F05FDE-E6D1-4801-9340-FDB28F8B8951}"/>
     <hyperlink ref="A485" r:id="rId2" display="https://www.codewars.com/kata/593c9175933500f33400003e" xr:uid="{BD093DC0-F85E-47F2-AD40-991767FDE3C7}"/>

</xml_diff>

<commit_message>
Review 6 Problems 4/27/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0754F81E-861C-4E50-AA90-11F179233E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA251EC-0A69-4C61-B309-44D6E9AD34C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (85)</t>
+      <t xml:space="preserve"> (86)</t>
     </r>
   </si>
 </sst>
@@ -9797,7 +9797,7 @@
       <c r="F252" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G252" s="47" t="s">
+      <c r="G252" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9820,7 +9820,7 @@
       <c r="F253" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G253" s="47" t="s">
+      <c r="G253" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9843,7 +9843,7 @@
       <c r="F254" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G254" s="47" t="s">
+      <c r="G254" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9866,7 +9866,7 @@
       <c r="F255" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G255" s="47" t="s">
+      <c r="G255" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviwed 5 Problems 4/28/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA251EC-0A69-4C61-B309-44D6E9AD34C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885A46E1-16E3-4CC3-A4D0-7B45BA982EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3706,9 +3706,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FF800000"/>
       <color rgb="FFAD8043"/>
       <color rgb="FF308729"/>
-      <color rgb="FF800000"/>
       <color rgb="FFEF89E8"/>
       <color rgb="FFB97EFA"/>
       <color rgb="FFEAF4EA"/>
@@ -9889,7 +9889,7 @@
       <c r="F256" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G256" s="47" t="s">
+      <c r="G256" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9912,7 +9912,7 @@
       <c r="F257" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G257" s="47" t="s">
+      <c r="G257" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9935,7 +9935,7 @@
       <c r="F258" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G258" s="47" t="s">
+      <c r="G258" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
       <c r="F259" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G259" s="47" t="s">
+      <c r="G259" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -9981,7 +9981,7 @@
       <c r="F260" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G260" s="47" t="s">
+      <c r="G260" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewd 5 Problems 4/29/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885A46E1-16E3-4CC3-A4D0-7B45BA982EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E3D667-4F08-42F4-8D06-45C89A258769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3706,11 +3706,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFB97EFA"/>
       <color rgb="FF800000"/>
       <color rgb="FFAD8043"/>
       <color rgb="FF308729"/>
       <color rgb="FFEF89E8"/>
-      <color rgb="FFB97EFA"/>
       <color rgb="FFEAF4EA"/>
       <color rgb="FFE1E0FE"/>
       <color rgb="FFFEE0E0"/>
@@ -10004,7 +10004,7 @@
       <c r="F261" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G261" s="47" t="s">
+      <c r="G261" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10027,7 +10027,7 @@
       <c r="F262" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G262" s="47" t="s">
+      <c r="G262" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10050,7 +10050,7 @@
       <c r="F263" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G263" s="47" t="s">
+      <c r="G263" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10073,7 +10073,7 @@
       <c r="F264" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G264" s="47" t="s">
+      <c r="G264" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10096,7 +10096,7 @@
       <c r="F265" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G265" s="47" t="s">
+      <c r="G265" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 5 Problems 4/30/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E3D667-4F08-42F4-8D06-45C89A258769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2427EA-4AB1-4D79-B5E4-951EA220AAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10119,7 +10119,7 @@
       <c r="F266" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G266" s="47" t="s">
+      <c r="G266" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10142,7 +10142,7 @@
       <c r="F267" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G267" s="47" t="s">
+      <c r="G267" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10165,7 +10165,7 @@
       <c r="F268" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G268" s="47" t="s">
+      <c r="G268" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10188,7 +10188,7 @@
       <c r="F269" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G269" s="47" t="s">
+      <c r="G269" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10211,7 +10211,7 @@
       <c r="F270" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G270" s="47" t="s">
+      <c r="G270" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 5 Problems 5/2/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2427EA-4AB1-4D79-B5E4-951EA220AAF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F519DA-CE77-436D-A454-5CD81430C10D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10234,7 +10234,7 @@
       <c r="F271" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G271" s="47" t="s">
+      <c r="G271" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10257,7 +10257,7 @@
       <c r="F272" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G272" s="47" t="s">
+      <c r="G272" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10280,7 +10280,7 @@
       <c r="F273" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G273" s="47" t="s">
+      <c r="G273" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Review 5 Problems In Same Day 5/2/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F519DA-CE77-436D-A454-5CD81430C10D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26781CB-17B9-46A7-9EE2-1A6BAB14AB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (86)</t>
+      <t xml:space="preserve"> (89)</t>
     </r>
   </si>
 </sst>
@@ -10303,7 +10303,7 @@
       <c r="F274" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G274" s="47" t="s">
+      <c r="G274" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10326,7 +10326,7 @@
       <c r="F275" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G275" s="47" t="s">
+      <c r="G275" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10349,7 +10349,7 @@
       <c r="F276" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G276" s="47" t="s">
+      <c r="G276" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10395,7 +10395,7 @@
       <c r="F278" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G278" s="47" t="s">
+      <c r="G278" s="34" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 6 Problems 5/4/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E26781CB-17B9-46A7-9EE2-1A6BAB14AB48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A0556B-36E5-490E-8064-BE2F9F3C391C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2544,7 +2544,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="73">
+  <fonts count="72">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2938,14 +2938,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FFFFC000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <i/>
       <sz val="12"/>
@@ -3251,9 +3243,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="52" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="151">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3412,7 +3404,7 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="61" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3436,10 +3428,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="70" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="69" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3494,9 +3486,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3512,7 +3501,7 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3527,10 +3516,10 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3557,7 +3546,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="51" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3597,7 +3586,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="53" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="52" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3609,6 +3598,9 @@
     <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="54" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3616,15 +3608,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="56" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="53" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3633,37 +3622,40 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="59" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="63" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="62" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="64" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="61" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="64" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="63" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="65" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="58" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="66" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3672,26 +3664,23 @@
     <xf numFmtId="0" fontId="67" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="68" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="69" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="68" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="70" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="45" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4489,7 +4478,7 @@
       </c>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="147" t="s">
+      <c r="A22" s="146" t="s">
         <v>14</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -5323,7 +5312,7 @@
       <c r="B58" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C58" s="148" t="s">
+      <c r="C58" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D58" s="10">
@@ -5346,7 +5335,7 @@
       <c r="B59" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C59" s="148" t="s">
+      <c r="C59" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D59" s="10">
@@ -5369,7 +5358,7 @@
       <c r="B60" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C60" s="148" t="s">
+      <c r="C60" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D60" s="10">
@@ -5392,7 +5381,7 @@
       <c r="B61" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C61" s="148" t="s">
+      <c r="C61" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D61" s="10">
@@ -5507,7 +5496,7 @@
       <c r="B66" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C66" s="148" t="s">
+      <c r="C66" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D66" s="10">
@@ -5530,7 +5519,7 @@
       <c r="B67" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C67" s="148" t="s">
+      <c r="C67" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D67" s="10">
@@ -7853,7 +7842,7 @@
       <c r="B168" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C168" s="148" t="s">
+      <c r="C168" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D168" s="10" t="s">
@@ -7876,7 +7865,7 @@
       <c r="B169" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C169" s="148" t="s">
+      <c r="C169" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D169" s="10" t="s">
@@ -7899,7 +7888,7 @@
       <c r="B170" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C170" s="148" t="s">
+      <c r="C170" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D170" s="10" t="s">
@@ -7922,7 +7911,7 @@
       <c r="B171" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C171" s="148" t="s">
+      <c r="C171" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D171" s="10" t="s">
@@ -7945,7 +7934,7 @@
       <c r="B172" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C172" s="148" t="s">
+      <c r="C172" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D172" s="10" t="s">
@@ -7968,7 +7957,7 @@
       <c r="B173" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C173" s="148" t="s">
+      <c r="C173" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D173" s="10" t="s">
@@ -7991,7 +7980,7 @@
       <c r="B174" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C174" s="148" t="s">
+      <c r="C174" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D174" s="10" t="s">
@@ -8014,7 +8003,7 @@
       <c r="B175" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C175" s="148" t="s">
+      <c r="C175" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D175" s="10" t="s">
@@ -8037,7 +8026,7 @@
       <c r="B176" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C176" s="148" t="s">
+      <c r="C176" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D176" s="10" t="s">
@@ -8083,7 +8072,7 @@
       <c r="B178" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C178" s="148" t="s">
+      <c r="C178" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D178" s="10" t="s">
@@ -8106,7 +8095,7 @@
       <c r="B179" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C179" s="148" t="s">
+      <c r="C179" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D179" s="10" t="s">
@@ -8129,7 +8118,7 @@
       <c r="B180" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C180" s="148" t="s">
+      <c r="C180" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D180" s="10" t="s">
@@ -8152,7 +8141,7 @@
       <c r="B181" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C181" s="148" t="s">
+      <c r="C181" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D181" s="10" t="s">
@@ -8175,7 +8164,7 @@
       <c r="B182" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C182" s="148" t="s">
+      <c r="C182" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D182" s="10" t="s">
@@ -8198,7 +8187,7 @@
       <c r="B183" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C183" s="148" t="s">
+      <c r="C183" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D183" s="10" t="s">
@@ -10418,7 +10407,7 @@
       <c r="F279" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G279" s="47" t="s">
+      <c r="G279" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10441,12 +10430,12 @@
       <c r="F280" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G280" s="47" t="s">
+      <c r="G280" s="9" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="281" spans="1:7">
-      <c r="A281" s="82" t="s">
+      <c r="A281" s="7" t="s">
         <v>247</v>
       </c>
       <c r="B281" s="22" t="s">
@@ -10464,7 +10453,7 @@
       <c r="F281" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G281" s="47" t="s">
+      <c r="G281" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10510,7 +10499,7 @@
       <c r="F283" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G283" s="47" t="s">
+      <c r="G283" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11165,7 +11154,7 @@
       <c r="B312" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C312" s="148" t="s">
+      <c r="C312" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D312" s="51">
@@ -11188,7 +11177,7 @@
       <c r="B313" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C313" s="148" t="s">
+      <c r="C313" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D313" s="51">
@@ -11257,7 +11246,7 @@
       <c r="B316" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C316" s="148" t="s">
+      <c r="C316" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D316" s="51">
@@ -12332,7 +12321,7 @@
       </c>
     </row>
     <row r="363" spans="1:7">
-      <c r="A363" s="83" t="s">
+      <c r="A363" s="82" t="s">
         <v>383</v>
       </c>
       <c r="B363" s="22" t="s">
@@ -12424,7 +12413,7 @@
       </c>
     </row>
     <row r="367" spans="1:7">
-      <c r="A367" s="84" t="s">
+      <c r="A367" s="83" t="s">
         <v>387</v>
       </c>
       <c r="B367" s="8" t="s">
@@ -12470,7 +12459,7 @@
       </c>
     </row>
     <row r="369" spans="1:7">
-      <c r="A369" s="84" t="s">
+      <c r="A369" s="83" t="s">
         <v>389</v>
       </c>
       <c r="B369" s="8" t="s">
@@ -12585,7 +12574,7 @@
       </c>
     </row>
     <row r="374" spans="1:7">
-      <c r="A374" s="85" t="s">
+      <c r="A374" s="84" t="s">
         <v>394</v>
       </c>
       <c r="B374" s="22" t="s">
@@ -12631,7 +12620,7 @@
       </c>
     </row>
     <row r="376" spans="1:7">
-      <c r="A376" s="86" t="s">
+      <c r="A376" s="85" t="s">
         <v>395</v>
       </c>
       <c r="B376" s="8" t="s">
@@ -12815,7 +12804,7 @@
       </c>
     </row>
     <row r="384" spans="1:7">
-      <c r="A384" s="87" t="s">
+      <c r="A384" s="86" t="s">
         <v>403</v>
       </c>
       <c r="B384" s="8" t="s">
@@ -12838,7 +12827,7 @@
       </c>
     </row>
     <row r="385" spans="1:8">
-      <c r="A385" s="88" t="s">
+      <c r="A385" s="87" t="s">
         <v>404</v>
       </c>
       <c r="B385" s="8" t="s">
@@ -12976,7 +12965,7 @@
       </c>
     </row>
     <row r="391" spans="1:8">
-      <c r="A391" s="89" t="s">
+      <c r="A391" s="88" t="s">
         <v>410</v>
       </c>
       <c r="B391" s="8" t="s">
@@ -13046,7 +13035,7 @@
       </c>
     </row>
     <row r="394" spans="1:8">
-      <c r="A394" s="90" t="s">
+      <c r="A394" s="89" t="s">
         <v>413</v>
       </c>
       <c r="B394" s="22" t="s">
@@ -13069,7 +13058,7 @@
       </c>
     </row>
     <row r="395" spans="1:8">
-      <c r="A395" s="91" t="s">
+      <c r="A395" s="90" t="s">
         <v>414</v>
       </c>
       <c r="B395" s="8" t="s">
@@ -13162,7 +13151,7 @@
       </c>
     </row>
     <row r="399" spans="1:8">
-      <c r="A399" s="92" t="s">
+      <c r="A399" s="91" t="s">
         <v>418</v>
       </c>
       <c r="B399" s="8" t="s">
@@ -13231,7 +13220,7 @@
       </c>
     </row>
     <row r="402" spans="1:8">
-      <c r="A402" s="93" t="s">
+      <c r="A402" s="92" t="s">
         <v>421</v>
       </c>
       <c r="B402" s="8" t="s">
@@ -13300,7 +13289,7 @@
       </c>
     </row>
     <row r="405" spans="1:8">
-      <c r="A405" s="94" t="s">
+      <c r="A405" s="93" t="s">
         <v>424</v>
       </c>
       <c r="B405" s="8" t="s">
@@ -13554,13 +13543,13 @@
       </c>
     </row>
     <row r="416" spans="1:8">
-      <c r="A416" s="95" t="s">
+      <c r="A416" s="94" t="s">
         <v>434</v>
       </c>
       <c r="B416" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C416" s="148" t="s">
+      <c r="C416" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D416" s="51">
@@ -13577,13 +13566,13 @@
       </c>
     </row>
     <row r="417" spans="1:7">
-      <c r="A417" s="96" t="s">
+      <c r="A417" s="95" t="s">
         <v>435</v>
       </c>
       <c r="B417" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C417" s="148" t="s">
+      <c r="C417" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D417" s="51">
@@ -13600,13 +13589,13 @@
       </c>
     </row>
     <row r="418" spans="1:7">
-      <c r="A418" s="85" t="s">
+      <c r="A418" s="84" t="s">
         <v>436</v>
       </c>
       <c r="B418" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C418" s="148" t="s">
+      <c r="C418" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D418" s="51">
@@ -13623,13 +13612,13 @@
       </c>
     </row>
     <row r="419" spans="1:7">
-      <c r="A419" s="90" t="s">
+      <c r="A419" s="89" t="s">
         <v>437</v>
       </c>
       <c r="B419" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C419" s="148" t="s">
+      <c r="C419" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D419" s="51">
@@ -13646,13 +13635,13 @@
       </c>
     </row>
     <row r="420" spans="1:7">
-      <c r="A420" s="97" t="s">
+      <c r="A420" s="96" t="s">
         <v>438</v>
       </c>
       <c r="B420" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C420" s="148" t="s">
+      <c r="C420" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D420" s="51">
@@ -13669,13 +13658,13 @@
       </c>
     </row>
     <row r="421" spans="1:7">
-      <c r="A421" s="98" t="s">
+      <c r="A421" s="97" t="s">
         <v>726</v>
       </c>
       <c r="B421" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C421" s="148" t="s">
+      <c r="C421" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D421" s="51">
@@ -13692,13 +13681,13 @@
       </c>
     </row>
     <row r="422" spans="1:7">
-      <c r="A422" s="95" t="s">
+      <c r="A422" s="94" t="s">
         <v>727</v>
       </c>
       <c r="B422" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C422" s="148" t="s">
+      <c r="C422" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D422" s="51">
@@ -13715,13 +13704,13 @@
       </c>
     </row>
     <row r="423" spans="1:7">
-      <c r="A423" s="99" t="s">
+      <c r="A423" s="98" t="s">
         <v>728</v>
       </c>
       <c r="B423" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C423" s="148" t="s">
+      <c r="C423" s="147" t="s">
         <v>13</v>
       </c>
       <c r="D423" s="51">
@@ -13738,7 +13727,7 @@
       </c>
     </row>
     <row r="424" spans="1:7">
-      <c r="A424" s="84" t="s">
+      <c r="A424" s="83" t="s">
         <v>439</v>
       </c>
       <c r="B424" s="8" t="s">
@@ -13761,7 +13750,7 @@
       </c>
     </row>
     <row r="425" spans="1:7">
-      <c r="A425" s="86" t="s">
+      <c r="A425" s="85" t="s">
         <v>440</v>
       </c>
       <c r="B425" s="8" t="s">
@@ -13830,7 +13819,7 @@
       </c>
     </row>
     <row r="428" spans="1:7">
-      <c r="A428" s="100" t="s">
+      <c r="A428" s="99" t="s">
         <v>443</v>
       </c>
       <c r="B428" s="4" t="s">
@@ -13853,7 +13842,7 @@
       </c>
     </row>
     <row r="429" spans="1:7">
-      <c r="A429" s="97" t="s">
+      <c r="A429" s="96" t="s">
         <v>444</v>
       </c>
       <c r="B429" s="8" t="s">
@@ -13968,7 +13957,7 @@
       </c>
     </row>
     <row r="434" spans="1:7">
-      <c r="A434" s="101" t="s">
+      <c r="A434" s="100" t="s">
         <v>449</v>
       </c>
       <c r="B434" s="4" t="s">
@@ -14037,7 +14026,7 @@
       </c>
     </row>
     <row r="437" spans="1:7">
-      <c r="A437" s="102" t="s">
+      <c r="A437" s="101" t="s">
         <v>453</v>
       </c>
       <c r="B437" s="4" t="s">
@@ -14083,7 +14072,7 @@
       </c>
     </row>
     <row r="439" spans="1:7">
-      <c r="A439" s="103" t="s">
+      <c r="A439" s="102" t="s">
         <v>455</v>
       </c>
       <c r="B439" s="8" t="s">
@@ -14106,7 +14095,7 @@
       </c>
     </row>
     <row r="440" spans="1:7">
-      <c r="A440" s="98" t="s">
+      <c r="A440" s="97" t="s">
         <v>456</v>
       </c>
       <c r="B440" s="8" t="s">
@@ -14152,7 +14141,7 @@
       </c>
     </row>
     <row r="442" spans="1:7">
-      <c r="A442" s="104" t="s">
+      <c r="A442" s="103" t="s">
         <v>458</v>
       </c>
       <c r="B442" s="8" t="s">
@@ -14198,7 +14187,7 @@
       </c>
     </row>
     <row r="444" spans="1:7">
-      <c r="A444" s="90" t="s">
+      <c r="A444" s="89" t="s">
         <v>460</v>
       </c>
       <c r="B444" s="8" t="s">
@@ -14221,7 +14210,7 @@
       </c>
     </row>
     <row r="445" spans="1:7">
-      <c r="A445" s="105" t="s">
+      <c r="A445" s="104" t="s">
         <v>461</v>
       </c>
       <c r="B445" s="8" t="s">
@@ -14290,7 +14279,7 @@
       </c>
     </row>
     <row r="448" spans="1:7">
-      <c r="A448" s="86" t="s">
+      <c r="A448" s="85" t="s">
         <v>464</v>
       </c>
       <c r="B448" s="8" t="s">
@@ -14313,7 +14302,7 @@
       </c>
     </row>
     <row r="449" spans="1:7">
-      <c r="A449" s="99" t="s">
+      <c r="A449" s="98" t="s">
         <v>465</v>
       </c>
       <c r="B449" s="8" t="s">
@@ -14336,7 +14325,7 @@
       </c>
     </row>
     <row r="450" spans="1:7">
-      <c r="A450" s="106" t="s">
+      <c r="A450" s="105" t="s">
         <v>466</v>
       </c>
       <c r="B450" s="8" t="s">
@@ -14382,7 +14371,7 @@
       </c>
     </row>
     <row r="452" spans="1:7">
-      <c r="A452" s="95" t="s">
+      <c r="A452" s="94" t="s">
         <v>468</v>
       </c>
       <c r="B452" s="8" t="s">
@@ -14405,7 +14394,7 @@
       </c>
     </row>
     <row r="453" spans="1:7">
-      <c r="A453" s="83" t="s">
+      <c r="A453" s="82" t="s">
         <v>469</v>
       </c>
       <c r="B453" s="8" t="s">
@@ -14474,7 +14463,7 @@
       </c>
     </row>
     <row r="456" spans="1:7">
-      <c r="A456" s="102" t="s">
+      <c r="A456" s="101" t="s">
         <v>472</v>
       </c>
       <c r="B456" s="8" t="s">
@@ -14497,7 +14486,7 @@
       </c>
     </row>
     <row r="457" spans="1:7">
-      <c r="A457" s="86" t="s">
+      <c r="A457" s="85" t="s">
         <v>473</v>
       </c>
       <c r="B457" s="8" t="s">
@@ -14520,7 +14509,7 @@
       </c>
     </row>
     <row r="458" spans="1:7">
-      <c r="A458" s="97" t="s">
+      <c r="A458" s="96" t="s">
         <v>474</v>
       </c>
       <c r="B458" s="8" t="s">
@@ -14543,7 +14532,7 @@
       </c>
     </row>
     <row r="459" spans="1:7">
-      <c r="A459" s="102" t="s">
+      <c r="A459" s="101" t="s">
         <v>475</v>
       </c>
       <c r="B459" s="8" t="s">
@@ -14589,7 +14578,7 @@
       </c>
     </row>
     <row r="461" spans="1:7">
-      <c r="A461" s="85" t="s">
+      <c r="A461" s="84" t="s">
         <v>477</v>
       </c>
       <c r="B461" s="8" t="s">
@@ -14612,7 +14601,7 @@
       </c>
     </row>
     <row r="462" spans="1:7">
-      <c r="A462" s="107" t="s">
+      <c r="A462" s="106" t="s">
         <v>478</v>
       </c>
       <c r="B462" s="8" t="s">
@@ -14658,7 +14647,7 @@
       </c>
     </row>
     <row r="464" spans="1:7">
-      <c r="A464" s="108" t="s">
+      <c r="A464" s="107" t="s">
         <v>480</v>
       </c>
       <c r="B464" s="8" t="s">
@@ -14704,7 +14693,7 @@
       </c>
     </row>
     <row r="466" spans="1:7">
-      <c r="A466" s="109" t="s">
+      <c r="A466" s="108" t="s">
         <v>482</v>
       </c>
       <c r="B466" s="8" t="s">
@@ -14727,7 +14716,7 @@
       </c>
     </row>
     <row r="467" spans="1:7">
-      <c r="A467" s="96" t="s">
+      <c r="A467" s="95" t="s">
         <v>483</v>
       </c>
       <c r="B467" s="8" t="s">
@@ -14750,7 +14739,7 @@
       </c>
     </row>
     <row r="468" spans="1:7">
-      <c r="A468" s="97" t="s">
+      <c r="A468" s="96" t="s">
         <v>484</v>
       </c>
       <c r="B468" s="8" t="s">
@@ -14773,7 +14762,7 @@
       </c>
     </row>
     <row r="469" spans="1:7">
-      <c r="A469" s="107" t="s">
+      <c r="A469" s="106" t="s">
         <v>485</v>
       </c>
       <c r="B469" s="8" t="s">
@@ -14819,7 +14808,7 @@
       </c>
     </row>
     <row r="471" spans="1:7">
-      <c r="A471" s="110" t="s">
+      <c r="A471" s="109" t="s">
         <v>487</v>
       </c>
       <c r="B471" s="8" t="s">
@@ -14980,7 +14969,7 @@
       </c>
     </row>
     <row r="478" spans="1:7">
-      <c r="A478" s="97" t="s">
+      <c r="A478" s="96" t="s">
         <v>494</v>
       </c>
       <c r="B478" s="8" t="s">
@@ -15026,7 +15015,7 @@
       </c>
     </row>
     <row r="480" spans="1:7">
-      <c r="A480" s="108" t="s">
+      <c r="A480" s="107" t="s">
         <v>496</v>
       </c>
       <c r="B480" s="8" t="s">
@@ -15095,7 +15084,7 @@
       </c>
     </row>
     <row r="483" spans="1:7">
-      <c r="A483" s="85" t="s">
+      <c r="A483" s="84" t="s">
         <v>499</v>
       </c>
       <c r="B483" s="8" t="s">
@@ -15118,7 +15107,7 @@
       </c>
     </row>
     <row r="484" spans="1:7">
-      <c r="A484" s="111" t="s">
+      <c r="A484" s="110" t="s">
         <v>500</v>
       </c>
       <c r="B484" s="8" t="s">
@@ -15141,7 +15130,7 @@
       </c>
     </row>
     <row r="485" spans="1:7">
-      <c r="A485" s="112" t="s">
+      <c r="A485" s="111" t="s">
         <v>501</v>
       </c>
       <c r="B485" s="8" t="s">
@@ -15164,7 +15153,7 @@
       </c>
     </row>
     <row r="486" spans="1:7">
-      <c r="A486" s="107" t="s">
+      <c r="A486" s="106" t="s">
         <v>502</v>
       </c>
       <c r="B486" s="8" t="s">
@@ -15210,7 +15199,7 @@
       </c>
     </row>
     <row r="488" spans="1:7">
-      <c r="A488" s="113" t="s">
+      <c r="A488" s="112" t="s">
         <v>504</v>
       </c>
       <c r="B488" s="8" t="s">
@@ -15256,7 +15245,7 @@
       </c>
     </row>
     <row r="490" spans="1:7">
-      <c r="A490" s="87" t="s">
+      <c r="A490" s="86" t="s">
         <v>506</v>
       </c>
       <c r="B490" s="8" t="s">
@@ -15279,7 +15268,7 @@
       </c>
     </row>
     <row r="491" spans="1:7">
-      <c r="A491" s="107" t="s">
+      <c r="A491" s="106" t="s">
         <v>507</v>
       </c>
       <c r="B491" s="8" t="s">
@@ -15302,7 +15291,7 @@
       </c>
     </row>
     <row r="492" spans="1:7">
-      <c r="A492" s="96" t="s">
+      <c r="A492" s="95" t="s">
         <v>508</v>
       </c>
       <c r="B492" s="8" t="s">
@@ -15348,7 +15337,7 @@
       </c>
     </row>
     <row r="494" spans="1:7">
-      <c r="A494" s="91" t="s">
+      <c r="A494" s="90" t="s">
         <v>510</v>
       </c>
       <c r="B494" s="8" t="s">
@@ -15371,7 +15360,7 @@
       </c>
     </row>
     <row r="495" spans="1:7">
-      <c r="A495" s="90" t="s">
+      <c r="A495" s="89" t="s">
         <v>511</v>
       </c>
       <c r="B495" s="8" t="s">
@@ -15440,7 +15429,7 @@
       </c>
     </row>
     <row r="498" spans="1:8">
-      <c r="A498" s="97" t="s">
+      <c r="A498" s="96" t="s">
         <v>514</v>
       </c>
       <c r="B498" s="8" t="s">
@@ -15463,7 +15452,7 @@
       </c>
     </row>
     <row r="499" spans="1:8">
-      <c r="A499" s="85" t="s">
+      <c r="A499" s="84" t="s">
         <v>515</v>
       </c>
       <c r="B499" s="8" t="s">
@@ -15486,7 +15475,7 @@
       </c>
     </row>
     <row r="500" spans="1:8">
-      <c r="A500" s="102" t="s">
+      <c r="A500" s="101" t="s">
         <v>516</v>
       </c>
       <c r="B500" s="8" t="s">
@@ -15509,7 +15498,7 @@
       </c>
     </row>
     <row r="501" spans="1:8">
-      <c r="A501" s="98" t="s">
+      <c r="A501" s="97" t="s">
         <v>517</v>
       </c>
       <c r="B501" s="8" t="s">
@@ -15532,7 +15521,7 @@
       </c>
     </row>
     <row r="502" spans="1:8">
-      <c r="A502" s="114" t="s">
+      <c r="A502" s="113" t="s">
         <v>518</v>
       </c>
       <c r="B502" s="8" t="s">
@@ -15555,7 +15544,7 @@
       </c>
     </row>
     <row r="503" spans="1:8">
-      <c r="A503" s="107" t="s">
+      <c r="A503" s="106" t="s">
         <v>520</v>
       </c>
       <c r="B503" s="8" t="s">
@@ -15578,7 +15567,7 @@
       </c>
     </row>
     <row r="504" spans="1:8">
-      <c r="A504" s="92" t="s">
+      <c r="A504" s="91" t="s">
         <v>519</v>
       </c>
       <c r="B504" s="8" t="s">
@@ -15601,7 +15590,7 @@
       </c>
     </row>
     <row r="505" spans="1:8">
-      <c r="A505" s="108" t="s">
+      <c r="A505" s="107" t="s">
         <v>521</v>
       </c>
       <c r="B505" s="8" t="s">
@@ -15625,7 +15614,7 @@
       <c r="H505" s="15"/>
     </row>
     <row r="506" spans="1:8">
-      <c r="A506" s="110" t="s">
+      <c r="A506" s="109" t="s">
         <v>522</v>
       </c>
       <c r="B506" s="8" t="s">
@@ -15648,7 +15637,7 @@
       </c>
     </row>
     <row r="507" spans="1:8">
-      <c r="A507" s="91" t="s">
+      <c r="A507" s="90" t="s">
         <v>523</v>
       </c>
       <c r="B507" s="8" t="s">
@@ -15694,7 +15683,7 @@
       </c>
     </row>
     <row r="509" spans="1:8">
-      <c r="A509" s="98" t="s">
+      <c r="A509" s="97" t="s">
         <v>524</v>
       </c>
       <c r="B509" s="8" t="s">
@@ -15809,7 +15798,7 @@
       </c>
     </row>
     <row r="514" spans="1:7">
-      <c r="A514" s="102" t="s">
+      <c r="A514" s="101" t="s">
         <v>529</v>
       </c>
       <c r="B514" s="8" t="s">
@@ -15832,7 +15821,7 @@
       </c>
     </row>
     <row r="515" spans="1:7">
-      <c r="A515" s="106" t="s">
+      <c r="A515" s="105" t="s">
         <v>530</v>
       </c>
       <c r="B515" s="8" t="s">
@@ -15855,7 +15844,7 @@
       </c>
     </row>
     <row r="516" spans="1:7">
-      <c r="A516" s="107" t="s">
+      <c r="A516" s="106" t="s">
         <v>531</v>
       </c>
       <c r="B516" s="8" t="s">
@@ -15878,7 +15867,7 @@
       </c>
     </row>
     <row r="517" spans="1:7">
-      <c r="A517" s="100" t="s">
+      <c r="A517" s="99" t="s">
         <v>532</v>
       </c>
       <c r="B517" s="8" t="s">
@@ -15924,7 +15913,7 @@
       </c>
     </row>
     <row r="519" spans="1:7">
-      <c r="A519" s="102" t="s">
+      <c r="A519" s="101" t="s">
         <v>534</v>
       </c>
       <c r="B519" s="8" t="s">
@@ -16039,7 +16028,7 @@
       </c>
     </row>
     <row r="524" spans="1:7">
-      <c r="A524" s="84" t="s">
+      <c r="A524" s="83" t="s">
         <v>539</v>
       </c>
       <c r="B524" s="8" t="s">
@@ -16154,7 +16143,7 @@
       </c>
     </row>
     <row r="529" spans="1:8">
-      <c r="A529" s="115" t="s">
+      <c r="A529" s="114" t="s">
         <v>544</v>
       </c>
       <c r="B529" s="8" t="s">
@@ -16200,7 +16189,7 @@
       </c>
     </row>
     <row r="531" spans="1:8">
-      <c r="A531" s="96" t="s">
+      <c r="A531" s="95" t="s">
         <v>546</v>
       </c>
       <c r="B531" s="8" t="s">
@@ -16221,10 +16210,10 @@
       <c r="G531" s="47" t="s">
         <v>263</v>
       </c>
-      <c r="H531" s="116"/>
+      <c r="H531" s="115"/>
     </row>
     <row r="532" spans="1:8">
-      <c r="A532" s="107" t="s">
+      <c r="A532" s="106" t="s">
         <v>547</v>
       </c>
       <c r="B532" s="8" t="s">
@@ -16270,7 +16259,7 @@
       </c>
     </row>
     <row r="534" spans="1:8">
-      <c r="A534" s="95" t="s">
+      <c r="A534" s="94" t="s">
         <v>549</v>
       </c>
       <c r="B534" s="8" t="s">
@@ -16385,7 +16374,7 @@
       </c>
     </row>
     <row r="539" spans="1:8">
-      <c r="A539" s="85" t="s">
+      <c r="A539" s="84" t="s">
         <v>554</v>
       </c>
       <c r="B539" s="8" t="s">
@@ -16408,7 +16397,7 @@
       </c>
     </row>
     <row r="540" spans="1:8">
-      <c r="A540" s="98" t="s">
+      <c r="A540" s="97" t="s">
         <v>555</v>
       </c>
       <c r="B540" s="8" t="s">
@@ -16454,7 +16443,7 @@
       </c>
     </row>
     <row r="542" spans="1:8">
-      <c r="A542" s="92" t="s">
+      <c r="A542" s="91" t="s">
         <v>556</v>
       </c>
       <c r="B542" s="8" t="s">
@@ -16477,7 +16466,7 @@
       </c>
     </row>
     <row r="543" spans="1:8">
-      <c r="A543" s="91" t="s">
+      <c r="A543" s="90" t="s">
         <v>558</v>
       </c>
       <c r="B543" s="8" t="s">
@@ -16638,7 +16627,7 @@
       </c>
     </row>
     <row r="550" spans="1:7">
-      <c r="A550" s="117" t="s">
+      <c r="A550" s="116" t="s">
         <v>565</v>
       </c>
       <c r="B550" s="8" t="s">
@@ -16661,7 +16650,7 @@
       </c>
     </row>
     <row r="551" spans="1:7">
-      <c r="A551" s="109" t="s">
+      <c r="A551" s="108" t="s">
         <v>566</v>
       </c>
       <c r="B551" s="8" t="s">
@@ -16684,7 +16673,7 @@
       </c>
     </row>
     <row r="552" spans="1:7">
-      <c r="A552" s="97" t="s">
+      <c r="A552" s="96" t="s">
         <v>567</v>
       </c>
       <c r="B552" s="8" t="s">
@@ -16776,7 +16765,7 @@
       </c>
     </row>
     <row r="556" spans="1:7">
-      <c r="A556" s="118" t="s">
+      <c r="A556" s="117" t="s">
         <v>571</v>
       </c>
       <c r="B556" s="8" t="s">
@@ -16868,7 +16857,7 @@
       </c>
     </row>
     <row r="560" spans="1:7">
-      <c r="A560" s="119" t="s">
+      <c r="A560" s="118" t="s">
         <v>575</v>
       </c>
       <c r="B560" s="8" t="s">
@@ -16891,7 +16880,7 @@
       </c>
     </row>
     <row r="561" spans="1:7">
-      <c r="A561" s="99" t="s">
+      <c r="A561" s="98" t="s">
         <v>576</v>
       </c>
       <c r="B561" s="8" t="s">
@@ -16914,7 +16903,7 @@
       </c>
     </row>
     <row r="562" spans="1:7">
-      <c r="A562" s="98" t="s">
+      <c r="A562" s="97" t="s">
         <v>577</v>
       </c>
       <c r="B562" s="8" t="s">
@@ -16937,7 +16926,7 @@
       </c>
     </row>
     <row r="563" spans="1:7">
-      <c r="A563" s="102" t="s">
+      <c r="A563" s="101" t="s">
         <v>578</v>
       </c>
       <c r="B563" s="8" t="s">
@@ -16960,7 +16949,7 @@
       </c>
     </row>
     <row r="564" spans="1:7">
-      <c r="A564" s="120" t="s">
+      <c r="A564" s="119" t="s">
         <v>579</v>
       </c>
       <c r="B564" s="8" t="s">
@@ -17006,7 +16995,7 @@
       </c>
     </row>
     <row r="566" spans="1:7">
-      <c r="A566" s="86" t="s">
+      <c r="A566" s="85" t="s">
         <v>581</v>
       </c>
       <c r="B566" s="8" t="s">
@@ -17029,7 +17018,7 @@
       </c>
     </row>
     <row r="567" spans="1:7">
-      <c r="A567" s="107" t="s">
+      <c r="A567" s="106" t="s">
         <v>582</v>
       </c>
       <c r="B567" s="8" t="s">
@@ -17075,7 +17064,7 @@
       </c>
     </row>
     <row r="569" spans="1:7">
-      <c r="A569" s="98" t="s">
+      <c r="A569" s="97" t="s">
         <v>584</v>
       </c>
       <c r="B569" s="8" t="s">
@@ -17121,7 +17110,7 @@
       </c>
     </row>
     <row r="571" spans="1:7">
-      <c r="A571" s="120" t="s">
+      <c r="A571" s="119" t="s">
         <v>586</v>
       </c>
       <c r="B571" s="8" t="s">
@@ -17282,7 +17271,7 @@
       </c>
     </row>
     <row r="578" spans="1:7">
-      <c r="A578" s="110" t="s">
+      <c r="A578" s="109" t="s">
         <v>593</v>
       </c>
       <c r="B578" s="8" t="s">
@@ -17305,7 +17294,7 @@
       </c>
     </row>
     <row r="579" spans="1:7">
-      <c r="A579" s="91" t="s">
+      <c r="A579" s="90" t="s">
         <v>594</v>
       </c>
       <c r="B579" s="8" t="s">
@@ -17328,7 +17317,7 @@
       </c>
     </row>
     <row r="580" spans="1:7">
-      <c r="A580" s="92" t="s">
+      <c r="A580" s="91" t="s">
         <v>595</v>
       </c>
       <c r="B580" s="8" t="s">
@@ -17466,7 +17455,7 @@
       </c>
     </row>
     <row r="586" spans="1:7">
-      <c r="A586" s="110" t="s">
+      <c r="A586" s="109" t="s">
         <v>600</v>
       </c>
       <c r="B586" s="8" t="s">
@@ -17489,7 +17478,7 @@
       </c>
     </row>
     <row r="587" spans="1:7">
-      <c r="A587" s="121" t="s">
+      <c r="A587" s="120" t="s">
         <v>601</v>
       </c>
       <c r="B587" s="8" t="s">
@@ -17535,7 +17524,7 @@
       </c>
     </row>
     <row r="589" spans="1:7">
-      <c r="A589" s="122" t="s">
+      <c r="A589" s="121" t="s">
         <v>603</v>
       </c>
       <c r="B589" s="8" t="s">
@@ -17558,7 +17547,7 @@
       </c>
     </row>
     <row r="590" spans="1:7">
-      <c r="A590" s="120" t="s">
+      <c r="A590" s="119" t="s">
         <v>604</v>
       </c>
       <c r="B590" s="8" t="s">
@@ -17581,7 +17570,7 @@
       </c>
     </row>
     <row r="591" spans="1:7">
-      <c r="A591" s="97" t="s">
+      <c r="A591" s="96" t="s">
         <v>605</v>
       </c>
       <c r="B591" s="8" t="s">
@@ -17604,7 +17593,7 @@
       </c>
     </row>
     <row r="592" spans="1:7">
-      <c r="A592" s="123" t="s">
+      <c r="A592" s="122" t="s">
         <v>606</v>
       </c>
       <c r="B592" s="8" t="s">
@@ -17627,7 +17616,7 @@
       </c>
     </row>
     <row r="593" spans="1:7">
-      <c r="A593" s="101" t="s">
+      <c r="A593" s="100" t="s">
         <v>607</v>
       </c>
       <c r="B593" s="8" t="s">
@@ -17650,7 +17639,7 @@
       </c>
     </row>
     <row r="594" spans="1:7">
-      <c r="A594" s="124" t="s">
+      <c r="A594" s="123" t="s">
         <v>608</v>
       </c>
       <c r="B594" s="8" t="s">
@@ -17673,7 +17662,7 @@
       </c>
     </row>
     <row r="595" spans="1:7">
-      <c r="A595" s="106" t="s">
+      <c r="A595" s="105" t="s">
         <v>609</v>
       </c>
       <c r="B595" s="8" t="s">
@@ -17719,7 +17708,7 @@
       </c>
     </row>
     <row r="597" spans="1:7">
-      <c r="A597" s="125" t="s">
+      <c r="A597" s="124" t="s">
         <v>611</v>
       </c>
       <c r="B597" s="8" t="s">
@@ -17811,7 +17800,7 @@
       </c>
     </row>
     <row r="601" spans="1:7">
-      <c r="A601" s="105" t="s">
+      <c r="A601" s="104" t="s">
         <v>615</v>
       </c>
       <c r="B601" s="8" t="s">
@@ -17834,7 +17823,7 @@
       </c>
     </row>
     <row r="602" spans="1:7">
-      <c r="A602" s="125" t="s">
+      <c r="A602" s="124" t="s">
         <v>617</v>
       </c>
       <c r="B602" s="8" t="s">
@@ -17857,7 +17846,7 @@
       </c>
     </row>
     <row r="603" spans="1:7">
-      <c r="A603" s="123" t="s">
+      <c r="A603" s="122" t="s">
         <v>616</v>
       </c>
       <c r="B603" s="8" t="s">
@@ -17926,7 +17915,7 @@
       </c>
     </row>
     <row r="606" spans="1:7">
-      <c r="A606" s="105" t="s">
+      <c r="A606" s="104" t="s">
         <v>620</v>
       </c>
       <c r="B606" s="8" t="s">
@@ -17949,7 +17938,7 @@
       </c>
     </row>
     <row r="607" spans="1:7">
-      <c r="A607" s="107" t="s">
+      <c r="A607" s="106" t="s">
         <v>621</v>
       </c>
       <c r="B607" s="8" t="s">
@@ -17972,7 +17961,7 @@
       </c>
     </row>
     <row r="608" spans="1:7">
-      <c r="A608" s="101" t="s">
+      <c r="A608" s="100" t="s">
         <v>622</v>
       </c>
       <c r="B608" s="8" t="s">
@@ -17995,7 +17984,7 @@
       </c>
     </row>
     <row r="609" spans="1:7">
-      <c r="A609" s="87" t="s">
+      <c r="A609" s="86" t="s">
         <v>623</v>
       </c>
       <c r="B609" s="8" t="s">
@@ -18018,7 +18007,7 @@
       </c>
     </row>
     <row r="610" spans="1:7">
-      <c r="A610" s="126" t="s">
+      <c r="A610" s="125" t="s">
         <v>624</v>
       </c>
       <c r="B610" s="8" t="s">
@@ -18041,7 +18030,7 @@
       </c>
     </row>
     <row r="611" spans="1:7">
-      <c r="A611" s="121" t="s">
+      <c r="A611" s="120" t="s">
         <v>625</v>
       </c>
       <c r="B611" s="8" t="s">
@@ -18087,7 +18076,7 @@
       </c>
     </row>
     <row r="613" spans="1:7">
-      <c r="A613" s="120" t="s">
+      <c r="A613" s="119" t="s">
         <v>627</v>
       </c>
       <c r="B613" s="8" t="s">
@@ -18110,7 +18099,7 @@
       </c>
     </row>
     <row r="614" spans="1:7">
-      <c r="A614" s="92" t="s">
+      <c r="A614" s="91" t="s">
         <v>628</v>
       </c>
       <c r="B614" s="8" t="s">
@@ -18156,7 +18145,7 @@
       </c>
     </row>
     <row r="616" spans="1:7">
-      <c r="A616" s="123" t="s">
+      <c r="A616" s="122" t="s">
         <v>630</v>
       </c>
       <c r="B616" s="8" t="s">
@@ -18179,7 +18168,7 @@
       </c>
     </row>
     <row r="617" spans="1:7">
-      <c r="A617" s="85" t="s">
+      <c r="A617" s="84" t="s">
         <v>631</v>
       </c>
       <c r="B617" s="8" t="s">
@@ -18202,7 +18191,7 @@
       </c>
     </row>
     <row r="618" spans="1:7">
-      <c r="A618" s="109" t="s">
+      <c r="A618" s="108" t="s">
         <v>632</v>
       </c>
       <c r="B618" s="8" t="s">
@@ -18248,7 +18237,7 @@
       </c>
     </row>
     <row r="620" spans="1:7">
-      <c r="A620" s="97" t="s">
+      <c r="A620" s="96" t="s">
         <v>634</v>
       </c>
       <c r="B620" s="8" t="s">
@@ -18294,7 +18283,7 @@
       </c>
     </row>
     <row r="622" spans="1:7">
-      <c r="A622" s="106" t="s">
+      <c r="A622" s="105" t="s">
         <v>636</v>
       </c>
       <c r="B622" s="8" t="s">
@@ -18340,7 +18329,7 @@
       </c>
     </row>
     <row r="624" spans="1:7">
-      <c r="A624" s="101" t="s">
+      <c r="A624" s="100" t="s">
         <v>637</v>
       </c>
       <c r="B624" s="8" t="s">
@@ -18386,7 +18375,7 @@
       </c>
     </row>
     <row r="626" spans="1:7">
-      <c r="A626" s="127" t="s">
+      <c r="A626" s="126" t="s">
         <v>639</v>
       </c>
       <c r="B626" s="8" t="s">
@@ -18409,7 +18398,7 @@
       </c>
     </row>
     <row r="627" spans="1:7">
-      <c r="A627" s="108" t="s">
+      <c r="A627" s="107" t="s">
         <v>640</v>
       </c>
       <c r="B627" s="8" t="s">
@@ -18432,7 +18421,7 @@
       </c>
     </row>
     <row r="628" spans="1:7">
-      <c r="A628" s="122" t="s">
+      <c r="A628" s="121" t="s">
         <v>641</v>
       </c>
       <c r="B628" s="8" t="s">
@@ -18478,7 +18467,7 @@
       </c>
     </row>
     <row r="630" spans="1:7">
-      <c r="A630" s="128" t="s">
+      <c r="A630" s="127" t="s">
         <v>643</v>
       </c>
       <c r="B630" s="8" t="s">
@@ -18524,7 +18513,7 @@
       </c>
     </row>
     <row r="632" spans="1:7">
-      <c r="A632" s="129" t="s">
+      <c r="A632" s="128" t="s">
         <v>646</v>
       </c>
       <c r="B632" s="8" t="s">
@@ -18593,7 +18582,7 @@
       </c>
     </row>
     <row r="635" spans="1:7">
-      <c r="A635" s="130" t="s">
+      <c r="A635" s="129" t="s">
         <v>649</v>
       </c>
       <c r="B635" s="8" t="s">
@@ -18616,7 +18605,7 @@
       </c>
     </row>
     <row r="636" spans="1:7">
-      <c r="A636" s="131" t="s">
+      <c r="A636" s="130" t="s">
         <v>650</v>
       </c>
       <c r="B636" s="8" t="s">
@@ -18639,7 +18628,7 @@
       </c>
     </row>
     <row r="637" spans="1:7">
-      <c r="A637" s="118" t="s">
+      <c r="A637" s="117" t="s">
         <v>651</v>
       </c>
       <c r="B637" s="8" t="s">
@@ -18662,7 +18651,7 @@
       </c>
     </row>
     <row r="638" spans="1:7">
-      <c r="A638" s="132" t="s">
+      <c r="A638" s="131" t="s">
         <v>652</v>
       </c>
       <c r="B638" s="8" t="s">
@@ -18685,7 +18674,7 @@
       </c>
     </row>
     <row r="639" spans="1:7">
-      <c r="A639" s="104" t="s">
+      <c r="A639" s="103" t="s">
         <v>653</v>
       </c>
       <c r="B639" s="8" t="s">
@@ -18731,7 +18720,7 @@
       </c>
     </row>
     <row r="641" spans="1:7">
-      <c r="A641" s="119" t="s">
+      <c r="A641" s="118" t="s">
         <v>655</v>
       </c>
       <c r="B641" s="8" t="s">
@@ -18754,7 +18743,7 @@
       </c>
     </row>
     <row r="642" spans="1:7">
-      <c r="A642" s="92" t="s">
+      <c r="A642" s="91" t="s">
         <v>657</v>
       </c>
       <c r="B642" s="8" t="s">
@@ -18777,7 +18766,7 @@
       </c>
     </row>
     <row r="643" spans="1:7">
-      <c r="A643" s="125" t="s">
+      <c r="A643" s="124" t="s">
         <v>658</v>
       </c>
       <c r="B643" s="8" t="s">
@@ -18800,7 +18789,7 @@
       </c>
     </row>
     <row r="644" spans="1:7">
-      <c r="A644" s="133" t="s">
+      <c r="A644" s="132" t="s">
         <v>659</v>
       </c>
       <c r="B644" s="8" t="s">
@@ -18823,7 +18812,7 @@
       </c>
     </row>
     <row r="645" spans="1:7">
-      <c r="A645" s="98" t="s">
+      <c r="A645" s="97" t="s">
         <v>660</v>
       </c>
       <c r="B645" s="8" t="s">
@@ -18869,7 +18858,7 @@
       </c>
     </row>
     <row r="647" spans="1:7">
-      <c r="A647" s="125" t="s">
+      <c r="A647" s="124" t="s">
         <v>662</v>
       </c>
       <c r="B647" s="8" t="s">
@@ -18892,7 +18881,7 @@
       </c>
     </row>
     <row r="648" spans="1:7">
-      <c r="A648" s="107" t="s">
+      <c r="A648" s="106" t="s">
         <v>663</v>
       </c>
       <c r="B648" s="8" t="s">
@@ -18984,7 +18973,7 @@
       </c>
     </row>
     <row r="652" spans="1:7">
-      <c r="A652" s="84" t="s">
+      <c r="A652" s="83" t="s">
         <v>667</v>
       </c>
       <c r="B652" s="8" t="s">
@@ -19007,7 +18996,7 @@
       </c>
     </row>
     <row r="653" spans="1:7">
-      <c r="A653" s="121" t="s">
+      <c r="A653" s="120" t="s">
         <v>668</v>
       </c>
       <c r="B653" s="8" t="s">
@@ -19053,7 +19042,7 @@
       </c>
     </row>
     <row r="655" spans="1:7">
-      <c r="A655" s="92" t="s">
+      <c r="A655" s="91" t="s">
         <v>670</v>
       </c>
       <c r="B655" s="8" t="s">
@@ -19122,7 +19111,7 @@
       </c>
     </row>
     <row r="658" spans="1:8">
-      <c r="A658" s="91" t="s">
+      <c r="A658" s="90" t="s">
         <v>673</v>
       </c>
       <c r="B658" s="8" t="s">
@@ -19166,10 +19155,10 @@
       <c r="G659" s="34" t="s">
         <v>263</v>
       </c>
-      <c r="H659" s="116"/>
+      <c r="H659" s="115"/>
     </row>
     <row r="660" spans="1:8">
-      <c r="A660" s="134" t="s">
+      <c r="A660" s="133" t="s">
         <v>675</v>
       </c>
       <c r="B660" s="8" t="s">
@@ -19215,7 +19204,7 @@
       </c>
     </row>
     <row r="662" spans="1:8">
-      <c r="A662" s="100" t="s">
+      <c r="A662" s="99" t="s">
         <v>677</v>
       </c>
       <c r="B662" s="8" t="s">
@@ -19238,7 +19227,7 @@
       </c>
     </row>
     <row r="663" spans="1:8">
-      <c r="A663" s="121" t="s">
+      <c r="A663" s="120" t="s">
         <v>678</v>
       </c>
       <c r="B663" s="8" t="s">
@@ -19261,7 +19250,7 @@
       </c>
     </row>
     <row r="664" spans="1:8">
-      <c r="A664" s="135" t="s">
+      <c r="A664" s="134" t="s">
         <v>679</v>
       </c>
       <c r="B664" s="8" t="s">
@@ -19284,7 +19273,7 @@
       </c>
     </row>
     <row r="665" spans="1:8">
-      <c r="A665" s="97" t="s">
+      <c r="A665" s="96" t="s">
         <v>680</v>
       </c>
       <c r="B665" s="8" t="s">
@@ -19307,7 +19296,7 @@
       </c>
     </row>
     <row r="666" spans="1:8">
-      <c r="A666" s="108" t="s">
+      <c r="A666" s="107" t="s">
         <v>743</v>
       </c>
       <c r="B666" s="8" t="s">
@@ -19353,7 +19342,7 @@
       </c>
     </row>
     <row r="668" spans="1:8">
-      <c r="A668" s="120" t="s">
+      <c r="A668" s="119" t="s">
         <v>682</v>
       </c>
       <c r="B668" s="8" t="s">
@@ -19376,7 +19365,7 @@
       </c>
     </row>
     <row r="669" spans="1:8">
-      <c r="A669" s="85" t="s">
+      <c r="A669" s="84" t="s">
         <v>683</v>
       </c>
       <c r="B669" s="8" t="s">
@@ -19422,7 +19411,7 @@
       </c>
     </row>
     <row r="671" spans="1:8">
-      <c r="A671" s="136" t="s">
+      <c r="A671" s="135" t="s">
         <v>685</v>
       </c>
       <c r="B671" s="8" t="s">
@@ -19468,7 +19457,7 @@
       </c>
     </row>
     <row r="673" spans="1:7">
-      <c r="A673" s="108" t="s">
+      <c r="A673" s="107" t="s">
         <v>687</v>
       </c>
       <c r="B673" s="8" t="s">
@@ -19491,7 +19480,7 @@
       </c>
     </row>
     <row r="674" spans="1:7">
-      <c r="A674" s="119" t="s">
+      <c r="A674" s="118" t="s">
         <v>688</v>
       </c>
       <c r="B674" s="8" t="s">
@@ -19514,7 +19503,7 @@
       </c>
     </row>
     <row r="675" spans="1:7">
-      <c r="A675" s="107" t="s">
+      <c r="A675" s="106" t="s">
         <v>689</v>
       </c>
       <c r="B675" s="8" t="s">
@@ -19537,7 +19526,7 @@
       </c>
     </row>
     <row r="676" spans="1:7">
-      <c r="A676" s="121" t="s">
+      <c r="A676" s="120" t="s">
         <v>690</v>
       </c>
       <c r="B676" s="8" t="s">
@@ -19560,7 +19549,7 @@
       </c>
     </row>
     <row r="677" spans="1:7">
-      <c r="A677" s="105" t="s">
+      <c r="A677" s="104" t="s">
         <v>691</v>
       </c>
       <c r="B677" s="8" t="s">
@@ -19583,7 +19572,7 @@
       </c>
     </row>
     <row r="678" spans="1:7" ht="16.5">
-      <c r="A678" s="137" t="s">
+      <c r="A678" s="136" t="s">
         <v>692</v>
       </c>
       <c r="B678" s="8" t="s">
@@ -19606,7 +19595,7 @@
       </c>
     </row>
     <row r="679" spans="1:7">
-      <c r="A679" s="100" t="s">
+      <c r="A679" s="99" t="s">
         <v>693</v>
       </c>
       <c r="B679" s="8" t="s">
@@ -19629,7 +19618,7 @@
       </c>
     </row>
     <row r="680" spans="1:7">
-      <c r="A680" s="138" t="s">
+      <c r="A680" s="137" t="s">
         <v>694</v>
       </c>
       <c r="B680" s="8" t="s">
@@ -19652,7 +19641,7 @@
       </c>
     </row>
     <row r="681" spans="1:7">
-      <c r="A681" s="84" t="s">
+      <c r="A681" s="83" t="s">
         <v>695</v>
       </c>
       <c r="B681" s="8" t="s">
@@ -19698,7 +19687,7 @@
       </c>
     </row>
     <row r="683" spans="1:7">
-      <c r="A683" s="139" t="s">
+      <c r="A683" s="138" t="s">
         <v>697</v>
       </c>
       <c r="B683" s="8" t="s">
@@ -19721,7 +19710,7 @@
       </c>
     </row>
     <row r="684" spans="1:7" ht="16.5">
-      <c r="A684" s="140" t="s">
+      <c r="A684" s="139" t="s">
         <v>698</v>
       </c>
       <c r="B684" s="8" t="s">
@@ -19744,7 +19733,7 @@
       </c>
     </row>
     <row r="685" spans="1:7" ht="16.5">
-      <c r="A685" s="141" t="s">
+      <c r="A685" s="140" t="s">
         <v>699</v>
       </c>
       <c r="B685" s="8" t="s">
@@ -19767,7 +19756,7 @@
       </c>
     </row>
     <row r="686" spans="1:7">
-      <c r="A686" s="109" t="s">
+      <c r="A686" s="108" t="s">
         <v>700</v>
       </c>
       <c r="B686" s="8" t="s">
@@ -19790,7 +19779,7 @@
       </c>
     </row>
     <row r="687" spans="1:7">
-      <c r="A687" s="89" t="s">
+      <c r="A687" s="88" t="s">
         <v>701</v>
       </c>
       <c r="B687" s="8" t="s">
@@ -19836,7 +19825,7 @@
       </c>
     </row>
     <row r="689" spans="1:7">
-      <c r="A689" s="100" t="s">
+      <c r="A689" s="99" t="s">
         <v>703</v>
       </c>
       <c r="B689" s="8" t="s">
@@ -19859,7 +19848,7 @@
       </c>
     </row>
     <row r="690" spans="1:7" ht="16.5">
-      <c r="A690" s="142" t="s">
+      <c r="A690" s="141" t="s">
         <v>704</v>
       </c>
       <c r="B690" s="8" t="s">
@@ -19928,7 +19917,7 @@
       </c>
     </row>
     <row r="693" spans="1:7">
-      <c r="A693" s="108" t="s">
+      <c r="A693" s="107" t="s">
         <v>707</v>
       </c>
       <c r="B693" s="8" t="s">
@@ -19997,7 +19986,7 @@
       </c>
     </row>
     <row r="696" spans="1:7">
-      <c r="A696" s="121" t="s">
+      <c r="A696" s="120" t="s">
         <v>710</v>
       </c>
       <c r="B696" s="8" t="s">
@@ -20112,7 +20101,7 @@
       </c>
     </row>
     <row r="701" spans="1:7">
-      <c r="A701" s="121" t="s">
+      <c r="A701" s="120" t="s">
         <v>715</v>
       </c>
       <c r="B701" s="8" t="s">
@@ -20158,7 +20147,7 @@
       </c>
     </row>
     <row r="703" spans="1:7">
-      <c r="A703" s="102" t="s">
+      <c r="A703" s="101" t="s">
         <v>717</v>
       </c>
       <c r="B703" s="8" t="s">
@@ -20204,7 +20193,7 @@
       </c>
     </row>
     <row r="705" spans="1:7">
-      <c r="A705" s="110" t="s">
+      <c r="A705" s="109" t="s">
         <v>719</v>
       </c>
       <c r="B705" s="8" t="s">
@@ -20273,7 +20262,7 @@
       </c>
     </row>
     <row r="708" spans="1:7">
-      <c r="A708" s="134" t="s">
+      <c r="A708" s="133" t="s">
         <v>722</v>
       </c>
       <c r="B708" s="8" t="s">
@@ -20365,7 +20354,7 @@
       </c>
     </row>
     <row r="712" spans="1:7">
-      <c r="A712" s="90" t="s">
+      <c r="A712" s="89" t="s">
         <v>732</v>
       </c>
       <c r="B712" s="8" t="s">
@@ -20503,7 +20492,7 @@
       </c>
     </row>
     <row r="718" spans="1:7">
-      <c r="A718" s="105" t="s">
+      <c r="A718" s="104" t="s">
         <v>747</v>
       </c>
       <c r="B718" s="8" t="s">
@@ -20572,7 +20561,7 @@
       </c>
     </row>
     <row r="721" spans="1:7">
-      <c r="A721" s="139" t="s">
+      <c r="A721" s="138" t="s">
         <v>750</v>
       </c>
       <c r="B721" s="8" t="s">
@@ -20595,7 +20584,7 @@
       </c>
     </row>
     <row r="722" spans="1:7">
-      <c r="A722" s="143" t="s">
+      <c r="A722" s="142" t="s">
         <v>751</v>
       </c>
       <c r="B722" s="8" t="s">
@@ -20664,7 +20653,7 @@
       </c>
     </row>
     <row r="725" spans="1:7">
-      <c r="A725" s="100" t="s">
+      <c r="A725" s="99" t="s">
         <v>754</v>
       </c>
       <c r="B725" s="8" t="s">
@@ -20687,7 +20676,7 @@
       </c>
     </row>
     <row r="726" spans="1:7">
-      <c r="A726" s="87" t="s">
+      <c r="A726" s="86" t="s">
         <v>755</v>
       </c>
       <c r="B726" s="8" t="s">
@@ -20710,7 +20699,7 @@
       </c>
     </row>
     <row r="727" spans="1:7">
-      <c r="A727" s="138" t="s">
+      <c r="A727" s="137" t="s">
         <v>756</v>
       </c>
       <c r="B727" s="8" t="s">
@@ -20733,7 +20722,7 @@
       </c>
     </row>
     <row r="728" spans="1:7">
-      <c r="A728" s="84" t="s">
+      <c r="A728" s="83" t="s">
         <v>757</v>
       </c>
       <c r="B728" s="8" t="s">
@@ -20756,7 +20745,7 @@
       </c>
     </row>
     <row r="729" spans="1:7">
-      <c r="A729" s="85" t="s">
+      <c r="A729" s="84" t="s">
         <v>758</v>
       </c>
       <c r="B729" s="8" t="s">
@@ -20779,7 +20768,7 @@
       </c>
     </row>
     <row r="730" spans="1:7">
-      <c r="A730" s="102" t="s">
+      <c r="A730" s="101" t="s">
         <v>759</v>
       </c>
       <c r="B730" s="8" t="s">
@@ -20802,7 +20791,7 @@
       </c>
     </row>
     <row r="731" spans="1:7">
-      <c r="A731" s="95" t="s">
+      <c r="A731" s="94" t="s">
         <v>760</v>
       </c>
       <c r="B731" s="8" t="s">
@@ -20825,7 +20814,7 @@
       </c>
     </row>
     <row r="732" spans="1:7">
-      <c r="A732" s="134" t="s">
+      <c r="A732" s="133" t="s">
         <v>761</v>
       </c>
       <c r="B732" s="8" t="s">
@@ -20848,7 +20837,7 @@
       </c>
     </row>
     <row r="733" spans="1:7">
-      <c r="A733" s="138" t="s">
+      <c r="A733" s="137" t="s">
         <v>762</v>
       </c>
       <c r="B733" s="8" t="s">
@@ -20871,7 +20860,7 @@
       </c>
     </row>
     <row r="734" spans="1:7">
-      <c r="A734" s="98" t="s">
+      <c r="A734" s="97" t="s">
         <v>763</v>
       </c>
       <c r="B734" s="8" t="s">
@@ -20894,7 +20883,7 @@
       </c>
     </row>
     <row r="735" spans="1:7">
-      <c r="A735" s="102" t="s">
+      <c r="A735" s="101" t="s">
         <v>764</v>
       </c>
       <c r="B735" s="8" t="s">
@@ -20963,7 +20952,7 @@
       </c>
     </row>
     <row r="738" spans="1:7">
-      <c r="A738" s="144" t="s">
+      <c r="A738" s="143" t="s">
         <v>767</v>
       </c>
       <c r="B738" s="8" t="s">
@@ -21009,7 +20998,7 @@
       </c>
     </row>
     <row r="740" spans="1:7">
-      <c r="A740" s="138" t="s">
+      <c r="A740" s="137" t="s">
         <v>769</v>
       </c>
       <c r="B740" s="8" t="s">
@@ -21193,7 +21182,7 @@
       </c>
     </row>
     <row r="748" spans="1:7">
-      <c r="A748" s="87" t="s">
+      <c r="A748" s="86" t="s">
         <v>777</v>
       </c>
       <c r="B748" s="8" t="s">
@@ -21285,42 +21274,42 @@
       </c>
     </row>
     <row r="752" spans="1:7">
-      <c r="A752" s="138"/>
+      <c r="A752" s="137"/>
     </row>
     <row r="753" spans="1:1">
-      <c r="A753" s="138"/>
+      <c r="A753" s="137"/>
     </row>
     <row r="754" spans="1:1">
-      <c r="A754" s="138"/>
+      <c r="A754" s="137"/>
     </row>
     <row r="755" spans="1:1">
-      <c r="A755" s="138"/>
+      <c r="A755" s="137"/>
     </row>
     <row r="756" spans="1:1">
-      <c r="A756" s="145"/>
+      <c r="A756" s="144"/>
     </row>
     <row r="757" spans="1:1" ht="18.5">
-      <c r="A757" s="149" t="s">
+      <c r="A757" s="148" t="s">
         <v>781</v>
       </c>
     </row>
     <row r="758" spans="1:1" ht="18.5">
-      <c r="A758" s="149" t="s">
+      <c r="A758" s="148" t="s">
         <v>782</v>
       </c>
     </row>
     <row r="759" spans="1:1" ht="18.5">
-      <c r="A759" s="149" t="s">
+      <c r="A759" s="148" t="s">
         <v>786</v>
       </c>
     </row>
     <row r="760" spans="1:1">
-      <c r="A760" s="150" t="s">
+      <c r="A760" s="149" t="s">
         <v>783</v>
       </c>
     </row>
     <row r="779" spans="1:6" ht="15.5">
-      <c r="A779" s="146"/>
+      <c r="A779" s="145"/>
       <c r="B779" s="8"/>
       <c r="C779" s="40"/>
       <c r="D779" s="51"/>
@@ -21328,7 +21317,7 @@
       <c r="F779" s="8"/>
     </row>
     <row r="780" spans="1:6" ht="15.5">
-      <c r="A780" s="146"/>
+      <c r="A780" s="145"/>
       <c r="B780" s="8"/>
       <c r="C780" s="40"/>
       <c r="D780" s="51"/>
@@ -21336,7 +21325,7 @@
       <c r="F780" s="8"/>
     </row>
     <row r="781" spans="1:6" ht="15.5">
-      <c r="A781" s="146"/>
+      <c r="A781" s="145"/>
       <c r="B781" s="8"/>
       <c r="C781" s="40"/>
       <c r="D781" s="51"/>
@@ -21344,7 +21333,7 @@
       <c r="F781" s="8"/>
     </row>
     <row r="782" spans="1:6" ht="15.5">
-      <c r="A782" s="146"/>
+      <c r="A782" s="145"/>
       <c r="B782" s="8"/>
       <c r="C782" s="40"/>
       <c r="D782" s="51"/>
@@ -21352,7 +21341,7 @@
       <c r="F782" s="8"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="72" type="noConversion"/>
+  <phoneticPr fontId="71" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A484" r:id="rId1" display="https://www.codewars.com/kata/57b68bc7b69bfc8209000307" xr:uid="{B3F05FDE-E6D1-4801-9340-FDB28F8B8951}"/>
     <hyperlink ref="A485" r:id="rId2" display="https://www.codewars.com/kata/593c9175933500f33400003e" xr:uid="{BD093DC0-F85E-47F2-AD40-991767FDE3C7}"/>

</xml_diff>

<commit_message>
Review 4 Problems Second Time Today 5/4/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A0556B-36E5-490E-8064-BE2F9F3C391C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756CC19D-B814-4627-8A6B-DA4DCAD03710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10522,7 +10522,7 @@
       <c r="F284" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G284" s="47" t="s">
+      <c r="G284" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10545,7 +10545,7 @@
       <c r="F285" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G285" s="47" t="s">
+      <c r="G285" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 5 Problems 5/5/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756CC19D-B814-4627-8A6B-DA4DCAD03710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0FBC055-6D1A-4FE6-8105-937F7A591009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10568,7 +10568,7 @@
       <c r="F286" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G286" s="47" t="s">
+      <c r="G286" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10591,7 +10591,7 @@
       <c r="F287" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G287" s="47" t="s">
+      <c r="G287" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10614,7 +10614,7 @@
       <c r="F288" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G288" s="47" t="s">
+      <c r="G288" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10660,7 +10660,7 @@
       <c r="F290" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G290" s="47" t="s">
+      <c r="G290" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review 4 Problems 5/6/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0FBC055-6D1A-4FE6-8105-937F7A591009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC40472-54AC-4218-B93A-2823CD881CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (89)</t>
+      <t xml:space="preserve"> (91)</t>
     </r>
   </si>
 </sst>
@@ -10683,7 +10683,7 @@
       <c r="F291" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G291" s="47" t="s">
+      <c r="G291" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10729,7 +10729,7 @@
       <c r="F293" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G293" s="47" t="s">
+      <c r="G293" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10752,7 +10752,7 @@
       <c r="F294" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G294" s="47" t="s">
+      <c r="G294" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10775,7 +10775,7 @@
       <c r="F295" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G295" s="47" t="s">
+      <c r="G295" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 3 Problems 5/6/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CC40472-54AC-4218-B93A-2823CD881CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6064ABF-F8BF-45F7-8AA7-CEBAC47CCEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -10798,7 +10798,7 @@
       <c r="F296" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G296" s="47" t="s">
+      <c r="G296" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       <c r="F297" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G297" s="47" t="s">
+      <c r="G297" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10844,7 +10844,7 @@
       <c r="F298" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G298" s="47" t="s">
+      <c r="G298" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review Problems Second Time Today 5/7/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6064ABF-F8BF-45F7-8AA7-CEBAC47CCEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5881C28-3B53-41D7-A223-D1CBDF40FFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (91)</t>
+      <t xml:space="preserve"> (89)</t>
     </r>
   </si>
 </sst>
@@ -3981,7 +3981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFC1C95-6620-4666-A840-FB4F0938EA8B}">
-  <dimension ref="A1:H782"/>
+  <dimension ref="A1:H784"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="79.7265625" style="2" customWidth="1"/>
@@ -10867,7 +10867,7 @@
       <c r="F299" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G299" s="34" t="s">
+      <c r="G299" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10936,7 +10936,7 @@
       <c r="F302" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G302" s="47" t="s">
+      <c r="G302" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10959,7 +10959,7 @@
       <c r="F303" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G303" s="47" t="s">
+      <c r="G303" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10982,7 +10982,7 @@
       <c r="F304" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G304" s="34" t="s">
+      <c r="G304" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -21286,43 +21286,33 @@
       <c r="A755" s="137"/>
     </row>
     <row r="756" spans="1:1">
-      <c r="A756" s="144"/>
-    </row>
-    <row r="757" spans="1:1" ht="18.5">
-      <c r="A757" s="148" t="s">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="758" spans="1:1" ht="18.5">
-      <c r="A758" s="148" t="s">
-        <v>782</v>
-      </c>
+      <c r="A756" s="137"/>
+    </row>
+    <row r="757" spans="1:1">
+      <c r="A757" s="137"/>
+    </row>
+    <row r="758" spans="1:1">
+      <c r="A758" s="144"/>
     </row>
     <row r="759" spans="1:1" ht="18.5">
       <c r="A759" s="148" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="760" spans="1:1" ht="18.5">
+      <c r="A760" s="148" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="761" spans="1:1" ht="18.5">
+      <c r="A761" s="148" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="760" spans="1:1">
-      <c r="A760" s="149" t="s">
+    <row r="762" spans="1:1">
+      <c r="A762" s="149" t="s">
         <v>783</v>
       </c>
-    </row>
-    <row r="779" spans="1:6" ht="15.5">
-      <c r="A779" s="145"/>
-      <c r="B779" s="8"/>
-      <c r="C779" s="40"/>
-      <c r="D779" s="51"/>
-      <c r="E779" s="20"/>
-      <c r="F779" s="8"/>
-    </row>
-    <row r="780" spans="1:6" ht="15.5">
-      <c r="A780" s="145"/>
-      <c r="B780" s="8"/>
-      <c r="C780" s="40"/>
-      <c r="D780" s="51"/>
-      <c r="E780" s="20"/>
-      <c r="F780" s="8"/>
     </row>
     <row r="781" spans="1:6" ht="15.5">
       <c r="A781" s="145"/>
@@ -21339,6 +21329,22 @@
       <c r="D782" s="51"/>
       <c r="E782" s="20"/>
       <c r="F782" s="8"/>
+    </row>
+    <row r="783" spans="1:6" ht="15.5">
+      <c r="A783" s="145"/>
+      <c r="B783" s="8"/>
+      <c r="C783" s="40"/>
+      <c r="D783" s="51"/>
+      <c r="E783" s="20"/>
+      <c r="F783" s="8"/>
+    </row>
+    <row r="784" spans="1:6" ht="15.5">
+      <c r="A784" s="145"/>
+      <c r="B784" s="8"/>
+      <c r="C784" s="40"/>
+      <c r="D784" s="51"/>
+      <c r="E784" s="20"/>
+      <c r="F784" s="8"/>
     </row>
   </sheetData>
   <phoneticPr fontId="71" type="noConversion"/>

</xml_diff>

<commit_message>
Review 1 Another Problem Today 5/7/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5881C28-3B53-41D7-A223-D1CBDF40FFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7DE024-3C29-4A1F-9935-66B251E79997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11005,7 +11005,7 @@
       <c r="F305" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G305" s="47" t="s">
+      <c r="G305" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 5 problems 5/11/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{186AE981-3BD3-4962-BD5C-2367FBE05FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E491F4-1C8A-4BE9-BD8E-9EF132BF287B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11120,7 +11120,7 @@
       <c r="F310" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G310" s="47" t="s">
+      <c r="G310" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11212,7 +11212,7 @@
       <c r="F314" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G314" s="47" t="s">
+      <c r="G314" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11281,7 +11281,7 @@
       <c r="F317" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G317" s="47" t="s">
+      <c r="G317" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11304,7 +11304,7 @@
       <c r="F318" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G318" s="47" t="s">
+      <c r="G318" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reveiwed 10 Problems 5/12/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9E491F4-1C8A-4BE9-BD8E-9EF132BF287B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54FF0475-B1DB-48A8-8B22-3F9AF873A1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (90)</t>
+      <t xml:space="preserve"> (92)</t>
     </r>
   </si>
 </sst>
@@ -11327,7 +11327,7 @@
       <c r="F319" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G319" s="47" t="s">
+      <c r="G319" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11350,7 +11350,7 @@
       <c r="F320" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G320" s="47" t="s">
+      <c r="G320" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11373,7 +11373,7 @@
       <c r="F321" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G321" s="47" t="s">
+      <c r="G321" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11396,7 +11396,7 @@
       <c r="F322" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G322" s="47" t="s">
+      <c r="G322" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11419,7 +11419,7 @@
       <c r="F323" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G323" s="47" t="s">
+      <c r="G323" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11442,7 +11442,7 @@
       <c r="F324" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G324" s="47" t="s">
+      <c r="G324" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11465,7 +11465,7 @@
       <c r="F325" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G325" s="47" t="s">
+      <c r="G325" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11488,7 +11488,7 @@
       <c r="F326" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G326" s="47" t="s">
+      <c r="G326" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11511,7 +11511,7 @@
       <c r="F327" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G327" s="47" t="s">
+      <c r="G327" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11534,7 +11534,7 @@
       <c r="F328" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G328" s="47" t="s">
+      <c r="G328" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 2 Problems 5/16/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E604F289-C56A-4605-B9D3-CB34E0E9CA1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02442E43-581D-4B8F-AAE9-E6B54C5BB628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11902,7 +11902,7 @@
       <c r="F344" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G344" s="47" t="s">
+      <c r="G344" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11925,7 +11925,7 @@
       <c r="F345" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G345" s="47" t="s">
+      <c r="G345" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 1 Problem 5/17/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02442E43-581D-4B8F-AAE9-E6B54C5BB628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A7378F-E82E-42E0-9A93-DC5D8F2750FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11948,7 +11948,7 @@
       <c r="F346" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G346" s="47" t="s">
+      <c r="G346" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 8 Problems 5/19/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A7378F-E82E-42E0-9A93-DC5D8F2750FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD4E3EB-2A8A-4982-AF7A-FB92738A80C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11971,7 +11971,7 @@
       <c r="F347" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G347" s="47" t="s">
+      <c r="G347" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -11994,7 +11994,7 @@
       <c r="F348" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="G348" s="47" t="s">
+      <c r="G348" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12017,7 +12017,7 @@
       <c r="F349" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G349" s="47" t="s">
+      <c r="G349" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12040,7 +12040,7 @@
       <c r="F350" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G350" s="47" t="s">
+      <c r="G350" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12063,7 +12063,7 @@
       <c r="F351" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G351" s="47" t="s">
+      <c r="G351" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12086,7 +12086,7 @@
       <c r="F352" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G352" s="47" t="s">
+      <c r="G352" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12109,7 +12109,7 @@
       <c r="F353" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G353" s="47" t="s">
+      <c r="G353" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12155,7 +12155,7 @@
       <c r="F355" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G355" s="47" t="s">
+      <c r="G355" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12178,7 +12178,7 @@
       <c r="F356" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G356" s="47" t="s">
+      <c r="G356" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12201,7 +12201,7 @@
       <c r="F357" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G357" s="47" t="s">
+      <c r="G357" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 2 Problems 5/20/206
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD4E3EB-2A8A-4982-AF7A-FB92738A80C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A209BF-9D6A-4746-B003-B4592A788CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2536,7 +2536,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (93)</t>
+      <t xml:space="preserve"> (94)</t>
     </r>
   </si>
 </sst>
@@ -12224,7 +12224,7 @@
       <c r="F358" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G358" s="47" t="s">
+      <c r="G358" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12247,7 +12247,7 @@
       <c r="F359" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G359" s="47" t="s">
+      <c r="G359" s="34" t="s">
         <v>263</v>
       </c>
     </row>
@@ -12270,7 +12270,7 @@
       <c r="F360" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G360" s="47" t="s">
+      <c r="G360" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 1 Problem 5/21/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A209BF-9D6A-4746-B003-B4592A788CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18534E8C-27B6-4ED9-8F62-50A5D0059276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12408,7 +12408,7 @@
       <c r="F366" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G366" s="47" t="s">
+      <c r="G366" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 1 Problem 7/13/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7FE563-E1B0-41DB-B85A-2133EA49E849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9680F6A2-2509-4A28-80AC-A9D6CBDF557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12523,7 +12523,7 @@
       <c r="F371" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G371" s="47" t="s">
+      <c r="G371" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 1 Problem 7/14/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9680F6A2-2509-4A28-80AC-A9D6CBDF557A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{273942BA-C7A8-468F-8BE2-404DEE4B9A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12546,7 +12546,7 @@
       <c r="F372" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="G372" s="47" t="s">
+      <c r="G372" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Reviewed 1 Problem 7/19/2026
</commit_message>
<xml_diff>
--- a/Problem Solving History.xlsx
+++ b/Problem Solving History.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Problem Solving\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67894FA1-1B58-474D-ACF3-80578B336C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF8EA5C-8D3B-48BE-8954-7F043B7190F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12638,7 +12638,7 @@
       <c r="F376" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G376" s="47" t="s">
+      <c r="G376" s="9" t="s">
         <v>263</v>
       </c>
     </row>

</xml_diff>